<commit_message>
Added analysis for carbon cost in the gas prices
</commit_message>
<xml_diff>
--- a/first_stage_optimization/lshp_operation.xlsx
+++ b/first_stage_optimization/lshp_operation.xlsx
@@ -439,10 +439,10 @@
         <v>288</v>
       </c>
       <c r="B2" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C2" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="3">
@@ -450,10 +450,10 @@
         <v>289</v>
       </c>
       <c r="B3" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C3" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="4">
@@ -461,10 +461,10 @@
         <v>290</v>
       </c>
       <c r="B4" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C4" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="5">
@@ -472,10 +472,10 @@
         <v>291</v>
       </c>
       <c r="B5" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C5" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="6">
@@ -483,10 +483,10 @@
         <v>292</v>
       </c>
       <c r="B6" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C6" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="7">
@@ -494,10 +494,10 @@
         <v>293</v>
       </c>
       <c r="B7" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C7" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="8">
@@ -505,10 +505,10 @@
         <v>294</v>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="9">
@@ -560,10 +560,10 @@
         <v>299</v>
       </c>
       <c r="B13" t="n">
-        <v>7571.621973941301</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C13" t="n">
-        <v>20883.24513659566</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="14">
@@ -571,10 +571,10 @@
         <v>300</v>
       </c>
       <c r="B14" t="n">
-        <v>4157.129133592324</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C14" t="n">
-        <v>11465.75292058619</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="15">
@@ -582,10 +582,10 @@
         <v>301</v>
       </c>
       <c r="B15" t="n">
-        <v>7859.845117504699</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C15" t="n">
-        <v>21678.19165951901</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="16">
@@ -593,10 +593,10 @@
         <v>302</v>
       </c>
       <c r="B16" t="n">
-        <v>3244.59692381376</v>
+        <v>7715.679075472789</v>
       </c>
       <c r="C16" t="n">
-        <v>8948.903307989189</v>
+        <v>21280.56816398705</v>
       </c>
     </row>
     <row r="17">
@@ -648,10 +648,10 @@
         <v>307</v>
       </c>
       <c r="B21" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C21" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="22">
@@ -659,10 +659,10 @@
         <v>308</v>
       </c>
       <c r="B22" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C22" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="23">
@@ -670,10 +670,10 @@
         <v>309</v>
       </c>
       <c r="B23" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C23" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="24">
@@ -681,10 +681,10 @@
         <v>310</v>
       </c>
       <c r="B24" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C24" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="25">
@@ -692,10 +692,10 @@
         <v>311</v>
       </c>
       <c r="B25" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C25" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="26">
@@ -703,10 +703,10 @@
         <v>312</v>
       </c>
       <c r="B26" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C26" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="27">
@@ -714,10 +714,10 @@
         <v>313</v>
       </c>
       <c r="B27" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C27" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="28">
@@ -725,10 +725,10 @@
         <v>314</v>
       </c>
       <c r="B28" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C28" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="29">
@@ -736,10 +736,10 @@
         <v>315</v>
       </c>
       <c r="B29" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C29" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="30">
@@ -747,10 +747,10 @@
         <v>316</v>
       </c>
       <c r="B30" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C30" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="31">
@@ -758,10 +758,10 @@
         <v>317</v>
       </c>
       <c r="B31" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C31" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="32">
@@ -769,10 +769,10 @@
         <v>318</v>
       </c>
       <c r="B32" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C32" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="33">
@@ -780,10 +780,10 @@
         <v>319</v>
       </c>
       <c r="B33" t="n">
-        <v>0</v>
+        <v>5061.248487878984</v>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>13959.3990869281</v>
       </c>
     </row>
     <row r="34">
@@ -813,10 +813,10 @@
         <v>322</v>
       </c>
       <c r="B36" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C36" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="37">
@@ -824,10 +824,10 @@
         <v>323</v>
       </c>
       <c r="B37" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C37" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="38">
@@ -835,10 +835,10 @@
         <v>324</v>
       </c>
       <c r="B38" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C38" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="39">
@@ -846,10 +846,10 @@
         <v>325</v>
       </c>
       <c r="B39" t="n">
-        <v>0</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="40">
@@ -857,10 +857,10 @@
         <v>326</v>
       </c>
       <c r="B40" t="n">
-        <v>0</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="41">
@@ -868,10 +868,10 @@
         <v>327</v>
       </c>
       <c r="B41" t="n">
-        <v>0</v>
+        <v>10522.31423963353</v>
       </c>
       <c r="C41" t="n">
-        <v>0</v>
+        <v>29021.53177044781</v>
       </c>
     </row>
     <row r="42">
@@ -901,10 +901,10 @@
         <v>330</v>
       </c>
       <c r="B44" t="n">
-        <v>1649.647793852731</v>
+        <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>4549.883682338455</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -912,10 +912,10 @@
         <v>331</v>
       </c>
       <c r="B45" t="n">
-        <v>2423.783616176349</v>
+        <v>6894.865767835377</v>
       </c>
       <c r="C45" t="n">
-        <v>6685.023049074291</v>
+        <v>19016.68790507215</v>
       </c>
     </row>
     <row r="46">
@@ -923,10 +923,10 @@
         <v>332</v>
       </c>
       <c r="B46" t="n">
-        <v>2606.87476649653</v>
+        <v>7077.956918155559</v>
       </c>
       <c r="C46" t="n">
-        <v>7190.005652225482</v>
+        <v>19521.67050822334</v>
       </c>
     </row>
     <row r="47">
@@ -934,10 +934,10 @@
         <v>333</v>
       </c>
       <c r="B47" t="n">
-        <v>3759.547892638409</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C47" t="n">
-        <v>10369.18648539864</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="48">
@@ -945,10 +945,10 @@
         <v>334</v>
       </c>
       <c r="B48" t="n">
-        <v>3913.606187237279</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C48" t="n">
-        <v>10794.09374338201</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="49">
@@ -956,10 +956,10 @@
         <v>335</v>
       </c>
       <c r="B49" t="n">
-        <v>2083.727200419131</v>
+        <v>6554.809352078159</v>
       </c>
       <c r="C49" t="n">
-        <v>5747.115489112803</v>
+        <v>18078.78034511066</v>
       </c>
     </row>
     <row r="50">
@@ -967,10 +967,10 @@
         <v>336</v>
       </c>
       <c r="B50" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C50" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="51">
@@ -978,10 +978,10 @@
         <v>337</v>
       </c>
       <c r="B51" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C51" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="52">
@@ -989,10 +989,10 @@
         <v>338</v>
       </c>
       <c r="B52" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C52" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="53">
@@ -1000,10 +1000,10 @@
         <v>339</v>
       </c>
       <c r="B53" t="n">
-        <v>6321.080014189263</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C53" t="n">
-        <v>17434.13286065532</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="54">
@@ -1011,10 +1011,10 @@
         <v>340</v>
       </c>
       <c r="B54" t="n">
-        <v>10997.65195901894</v>
+        <v>9400.398830393617</v>
       </c>
       <c r="C54" t="n">
-        <v>30332.55788225838</v>
+        <v>25927.18361171565</v>
       </c>
     </row>
     <row r="55">
@@ -1022,10 +1022,10 @@
         <v>341</v>
       </c>
       <c r="B55" t="n">
-        <v>5420.552036878907</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C55" t="n">
-        <v>14950.39204960349</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="56">
@@ -1220,10 +1220,10 @@
         <v>359</v>
       </c>
       <c r="B73" t="n">
-        <v>6228.763502302742</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C73" t="n">
-        <v>17179.51524312018</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="74">
@@ -1231,10 +1231,10 @@
         <v>360</v>
       </c>
       <c r="B74" t="n">
-        <v>5821.15015514865</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C74" t="n">
-        <v>16055.27931601456</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="75">
@@ -1242,10 +1242,10 @@
         <v>361</v>
       </c>
       <c r="B75" t="n">
-        <v>5809.795287589211</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C75" t="n">
-        <v>16023.96152392808</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="76">
@@ -1253,10 +1253,10 @@
         <v>362</v>
       </c>
       <c r="B76" t="n">
-        <v>5911.932054259483</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C76" t="n">
-        <v>16305.66432726075</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="77">
@@ -1264,10 +1264,10 @@
         <v>363</v>
       </c>
       <c r="B77" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C77" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="78">
@@ -1275,10 +1275,10 @@
         <v>364</v>
       </c>
       <c r="B78" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C78" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="79">
@@ -1286,10 +1286,10 @@
         <v>365</v>
       </c>
       <c r="B79" t="n">
-        <v>7754.904030281272</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C79" t="n">
-        <v>21388.75427649459</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="80">
@@ -1297,10 +1297,10 @@
         <v>366</v>
       </c>
       <c r="B80" t="n">
-        <v>9198.907302094618</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C80" t="n">
-        <v>25371.45103646335</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="81">
@@ -1374,10 +1374,10 @@
         <v>373</v>
       </c>
       <c r="B87" t="n">
-        <v>5684.661918074331</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C87" t="n">
-        <v>15678.8319282693</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="88">
@@ -1462,10 +1462,10 @@
         <v>381</v>
       </c>
       <c r="B95" t="n">
-        <v>0</v>
+        <v>1622.479896434131</v>
       </c>
       <c r="C95" t="n">
-        <v>0</v>
+        <v>4474.952067475599</v>
       </c>
     </row>
     <row r="96">
@@ -1473,10 +1473,10 @@
         <v>382</v>
       </c>
       <c r="B96" t="n">
-        <v>0</v>
+        <v>3756.082560895171</v>
       </c>
       <c r="C96" t="n">
-        <v>0</v>
+        <v>10359.62877470961</v>
       </c>
     </row>
     <row r="97">
@@ -1484,10 +1484,10 @@
         <v>383</v>
       </c>
       <c r="B97" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C97" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="98">
@@ -1495,10 +1495,10 @@
         <v>384</v>
       </c>
       <c r="B98" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C98" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="99">
@@ -1506,10 +1506,10 @@
         <v>385</v>
       </c>
       <c r="B99" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C99" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="100">
@@ -1517,10 +1517,10 @@
         <v>386</v>
       </c>
       <c r="B100" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C100" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="101">
@@ -1528,10 +1528,10 @@
         <v>387</v>
       </c>
       <c r="B101" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C101" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="102">
@@ -1539,10 +1539,10 @@
         <v>388</v>
       </c>
       <c r="B102" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C102" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="103">
@@ -1550,10 +1550,10 @@
         <v>389</v>
       </c>
       <c r="B103" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C103" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="104">
@@ -1561,10 +1561,10 @@
         <v>390</v>
       </c>
       <c r="B104" t="n">
-        <v>3801.67068790515</v>
+        <v>7837.206172529511</v>
       </c>
       <c r="C104" t="n">
-        <v>10485.36511428707</v>
+        <v>21615.75132121661</v>
       </c>
     </row>
     <row r="105">
@@ -1605,10 +1605,10 @@
         <v>394</v>
       </c>
       <c r="B108" t="n">
-        <v>0</v>
+        <v>2345.250100787285</v>
       </c>
       <c r="C108" t="n">
-        <v>0</v>
+        <v>6468.420231480806</v>
       </c>
     </row>
     <row r="109">
@@ -1627,10 +1627,10 @@
         <v>396</v>
       </c>
       <c r="B110" t="n">
-        <v>10361.8771713293</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C110" t="n">
-        <v>28579.03125498031</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="111">
@@ -1638,10 +1638,10 @@
         <v>397</v>
       </c>
       <c r="B111" t="n">
-        <v>9692.899210867357</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C111" t="n">
-        <v>26733.92715609799</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="112">
@@ -1715,10 +1715,10 @@
         <v>404</v>
       </c>
       <c r="B118" t="n">
-        <v>0</v>
+        <v>2696.459230950215</v>
       </c>
       <c r="C118" t="n">
-        <v>0</v>
+        <v>7437.088026128404</v>
       </c>
     </row>
     <row r="119">
@@ -1726,10 +1726,10 @@
         <v>405</v>
       </c>
       <c r="B119" t="n">
-        <v>0</v>
+        <v>4950.369843695064</v>
       </c>
       <c r="C119" t="n">
-        <v>0</v>
+        <v>13653.58536367629</v>
       </c>
     </row>
     <row r="120">
@@ -1737,10 +1737,10 @@
         <v>406</v>
       </c>
       <c r="B120" t="n">
-        <v>2140.480629651258</v>
+        <v>6176.01611427562</v>
       </c>
       <c r="C120" t="n">
-        <v>5903.646781757358</v>
+        <v>17034.0329886869</v>
       </c>
     </row>
     <row r="121">
@@ -1748,10 +1748,10 @@
         <v>407</v>
       </c>
       <c r="B121" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C121" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="122">
@@ -1759,10 +1759,10 @@
         <v>408</v>
       </c>
       <c r="B122" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C122" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="123">
@@ -1770,10 +1770,10 @@
         <v>409</v>
       </c>
       <c r="B123" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C123" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="124">
@@ -1781,10 +1781,10 @@
         <v>410</v>
       </c>
       <c r="B124" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C124" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="125">
@@ -1792,10 +1792,10 @@
         <v>411</v>
       </c>
       <c r="B125" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C125" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="126">
@@ -1803,10 +1803,10 @@
         <v>412</v>
       </c>
       <c r="B126" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C126" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="127">
@@ -1814,10 +1814,10 @@
         <v>413</v>
       </c>
       <c r="B127" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C127" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="128">
@@ -1825,10 +1825,10 @@
         <v>414</v>
       </c>
       <c r="B128" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C128" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="129">
@@ -1836,10 +1836,10 @@
         <v>415</v>
       </c>
       <c r="B129" t="n">
-        <v>8426.964116154217</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C129" t="n">
-        <v>23242.35916698025</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="130">
@@ -1847,10 +1847,10 @@
         <v>416</v>
       </c>
       <c r="B130" t="n">
-        <v>8593.836862446151</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C130" t="n">
-        <v>23702.60988729155</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="131">
@@ -1858,10 +1858,10 @@
         <v>417</v>
       </c>
       <c r="B131" t="n">
-        <v>8604.394097444776</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C131" t="n">
-        <v>23731.72773379785</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="132">
@@ -1869,10 +1869,10 @@
         <v>418</v>
       </c>
       <c r="B132" t="n">
-        <v>6674.542034261469</v>
+        <v>10710.07751888583</v>
       </c>
       <c r="C132" t="n">
-        <v>18409.01433744435</v>
+        <v>29539.40054437389</v>
       </c>
     </row>
     <row r="133">
@@ -1880,10 +1880,10 @@
         <v>419</v>
       </c>
       <c r="B133" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C133" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="134">
@@ -1891,10 +1891,10 @@
         <v>420</v>
       </c>
       <c r="B134" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C134" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="135">
@@ -1902,10 +1902,10 @@
         <v>421</v>
       </c>
       <c r="B135" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C135" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="136">
@@ -1913,10 +1913,10 @@
         <v>422</v>
       </c>
       <c r="B136" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C136" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="137">
@@ -1924,10 +1924,10 @@
         <v>423</v>
       </c>
       <c r="B137" t="n">
-        <v>0</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C137" t="n">
-        <v>0</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="138">
@@ -1935,10 +1935,10 @@
         <v>424</v>
       </c>
       <c r="B138" t="n">
-        <v>0</v>
+        <v>4081.108700781916</v>
       </c>
       <c r="C138" t="n">
-        <v>0</v>
+        <v>11256.0814209744</v>
       </c>
     </row>
     <row r="139">
@@ -1946,10 +1946,10 @@
         <v>425</v>
       </c>
       <c r="B139" t="n">
-        <v>0</v>
+        <v>5535.111192715002</v>
       </c>
       <c r="C139" t="n">
-        <v>0</v>
+        <v>15266.35696996009</v>
       </c>
     </row>
     <row r="140">
@@ -1957,10 +1957,10 @@
         <v>426</v>
       </c>
       <c r="B140" t="n">
-        <v>0</v>
+        <v>6538.550852195971</v>
       </c>
       <c r="C140" t="n">
-        <v>0</v>
+        <v>18033.93787413659</v>
       </c>
     </row>
     <row r="141">
@@ -1968,10 +1968,10 @@
         <v>427</v>
       </c>
       <c r="B141" t="n">
-        <v>0</v>
+        <v>6437.462881180372</v>
       </c>
       <c r="C141" t="n">
-        <v>0</v>
+        <v>17755.1277478063</v>
       </c>
     </row>
     <row r="142">
@@ -1979,10 +1979,10 @@
         <v>428</v>
       </c>
       <c r="B142" t="n">
-        <v>2029.366833690533</v>
+        <v>6064.902318314894</v>
       </c>
       <c r="C142" t="n">
-        <v>5597.184487800856</v>
+        <v>16727.5706947304</v>
       </c>
     </row>
     <row r="143">
@@ -1990,10 +1990,10 @@
         <v>429</v>
       </c>
       <c r="B143" t="n">
-        <v>2514.057212889899</v>
+        <v>6549.592697514261</v>
       </c>
       <c r="C143" t="n">
-        <v>6934.006114528354</v>
+        <v>18064.3923214579</v>
       </c>
     </row>
     <row r="144">
@@ -2001,10 +2001,10 @@
         <v>430</v>
       </c>
       <c r="B144" t="n">
-        <v>1719.1410707326</v>
+        <v>5754.676555356961</v>
       </c>
       <c r="C144" t="n">
-        <v>4741.55267234116</v>
+        <v>15871.9388792707</v>
       </c>
     </row>
     <row r="145">
@@ -2012,10 +2012,10 @@
         <v>431</v>
       </c>
       <c r="B145" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C145" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="146">
@@ -2023,10 +2023,10 @@
         <v>432</v>
       </c>
       <c r="B146" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C146" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="147">
@@ -2034,10 +2034,10 @@
         <v>433</v>
       </c>
       <c r="B147" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C147" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="148">
@@ -2045,10 +2045,10 @@
         <v>434</v>
       </c>
       <c r="B148" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C148" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="149">
@@ -2056,10 +2056,10 @@
         <v>435</v>
       </c>
       <c r="B149" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C149" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="150">
@@ -2067,10 +2067,10 @@
         <v>436</v>
       </c>
       <c r="B150" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C150" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="151">
@@ -2078,10 +2078,10 @@
         <v>437</v>
       </c>
       <c r="B151" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C151" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="152">
@@ -2089,10 +2089,10 @@
         <v>438</v>
       </c>
       <c r="B152" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C152" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="153">
@@ -2100,10 +2100,10 @@
         <v>439</v>
       </c>
       <c r="B153" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C153" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="154">
@@ -2111,10 +2111,10 @@
         <v>440</v>
       </c>
       <c r="B154" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C154" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="155">
@@ -2122,10 +2122,10 @@
         <v>441</v>
       </c>
       <c r="B155" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C155" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="156">
@@ -2133,10 +2133,10 @@
         <v>442</v>
       </c>
       <c r="B156" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C156" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="157">
@@ -2144,10 +2144,10 @@
         <v>443</v>
       </c>
       <c r="B157" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C157" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="158">
@@ -2155,10 +2155,10 @@
         <v>444</v>
       </c>
       <c r="B158" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C158" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="159">
@@ -2166,10 +2166,10 @@
         <v>445</v>
       </c>
       <c r="B159" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C159" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="160">
@@ -2177,10 +2177,10 @@
         <v>446</v>
       </c>
       <c r="B160" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C160" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="161">
@@ -2188,10 +2188,10 @@
         <v>447</v>
       </c>
       <c r="B161" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C161" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="162">
@@ -2221,10 +2221,10 @@
         <v>450</v>
       </c>
       <c r="B164" t="n">
-        <v>0</v>
+        <v>1644.834349911096</v>
       </c>
       <c r="C164" t="n">
-        <v>0</v>
+        <v>4536.607751483694</v>
       </c>
     </row>
     <row r="165">
@@ -2232,10 +2232,10 @@
         <v>451</v>
       </c>
       <c r="B165" t="n">
-        <v>0</v>
+        <v>3205.01860376423</v>
       </c>
       <c r="C165" t="n">
-        <v>0</v>
+        <v>8839.742580930499</v>
       </c>
     </row>
     <row r="166">
@@ -2243,10 +2243,10 @@
         <v>452</v>
       </c>
       <c r="B166" t="n">
-        <v>1649.647793852731</v>
+        <v>4927.983410894259</v>
       </c>
       <c r="C166" t="n">
-        <v>4549.883682338455</v>
+        <v>13591.84147768699</v>
       </c>
     </row>
     <row r="167">
@@ -2254,10 +2254,10 @@
         <v>453</v>
       </c>
       <c r="B167" t="n">
-        <v>3191.012512059943</v>
+        <v>7226.547996684305</v>
       </c>
       <c r="C167" t="n">
-        <v>8801.112463437457</v>
+        <v>19931.498670367</v>
       </c>
     </row>
     <row r="168">
@@ -2265,10 +2265,10 @@
         <v>454</v>
       </c>
       <c r="B168" t="n">
-        <v>5125.049000201142</v>
+        <v>9160.584484825504</v>
       </c>
       <c r="C168" t="n">
-        <v>14135.36689716077</v>
+        <v>25265.75310409031</v>
       </c>
     </row>
     <row r="169">
@@ -2276,10 +2276,10 @@
         <v>455</v>
       </c>
       <c r="B169" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C169" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="170">
@@ -2287,10 +2287,10 @@
         <v>456</v>
       </c>
       <c r="B170" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C170" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="171">
@@ -2298,10 +2298,10 @@
         <v>457</v>
       </c>
       <c r="B171" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C171" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="172">
@@ -2309,10 +2309,10 @@
         <v>458</v>
       </c>
       <c r="B172" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C172" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="173">
@@ -2320,10 +2320,10 @@
         <v>459</v>
       </c>
       <c r="B173" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C173" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="174">
@@ -2331,10 +2331,10 @@
         <v>460</v>
       </c>
       <c r="B174" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C174" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="175">
@@ -2342,10 +2342,10 @@
         <v>461</v>
       </c>
       <c r="B175" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C175" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="176">
@@ -2353,10 +2353,10 @@
         <v>462</v>
       </c>
       <c r="B176" t="n">
-        <v>6293.008293438715</v>
+        <v>10328.54377806308</v>
       </c>
       <c r="C176" t="n">
-        <v>17356.70841608356</v>
+        <v>28487.09462301311</v>
       </c>
     </row>
     <row r="177">
@@ -2518,10 +2518,10 @@
         <v>477</v>
       </c>
       <c r="B191" t="n">
-        <v>0</v>
+        <v>2695.174524152985</v>
       </c>
       <c r="C191" t="n">
-        <v>0</v>
+        <v>7433.544684019202</v>
       </c>
     </row>
     <row r="192">
@@ -2529,10 +2529,10 @@
         <v>478</v>
       </c>
       <c r="B192" t="n">
-        <v>0</v>
+        <v>3756.082560895171</v>
       </c>
       <c r="C192" t="n">
-        <v>0</v>
+        <v>10359.62877470961</v>
       </c>
     </row>
     <row r="193">
@@ -2540,10 +2540,10 @@
         <v>479</v>
       </c>
       <c r="B193" t="n">
-        <v>0</v>
+        <v>4403.242377510923</v>
       </c>
       <c r="C193" t="n">
-        <v>0</v>
+        <v>12144.55638195861</v>
       </c>
     </row>
     <row r="194">
@@ -2551,10 +2551,10 @@
         <v>480</v>
       </c>
       <c r="B194" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C194" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="195">
@@ -2562,10 +2562,10 @@
         <v>481</v>
       </c>
       <c r="B195" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C195" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="196">
@@ -2573,10 +2573,10 @@
         <v>482</v>
       </c>
       <c r="B196" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C196" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="197">
@@ -2584,10 +2584,10 @@
         <v>483</v>
       </c>
       <c r="B197" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C197" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="198">
@@ -2595,10 +2595,10 @@
         <v>484</v>
       </c>
       <c r="B198" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C198" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="199">
@@ -2606,10 +2606,10 @@
         <v>485</v>
       </c>
       <c r="B199" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C199" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="200">
@@ -2617,10 +2617,10 @@
         <v>486</v>
       </c>
       <c r="B200" t="n">
-        <v>6293.008293438715</v>
+        <v>10328.54377806308</v>
       </c>
       <c r="C200" t="n">
-        <v>17356.70841608356</v>
+        <v>28487.09462301311</v>
       </c>
     </row>
     <row r="201">
@@ -2628,10 +2628,10 @@
         <v>487</v>
       </c>
       <c r="B201" t="n">
-        <v>0</v>
+        <v>10026.99388425181</v>
       </c>
       <c r="C201" t="n">
-        <v>0</v>
+        <v>27655.3916701916</v>
       </c>
     </row>
     <row r="202">
@@ -2771,10 +2771,10 @@
         <v>500</v>
       </c>
       <c r="B214" t="n">
-        <v>0</v>
+        <v>2696.459230950215</v>
       </c>
       <c r="C214" t="n">
-        <v>0</v>
+        <v>7437.088026128404</v>
       </c>
     </row>
     <row r="215">
@@ -2782,10 +2782,10 @@
         <v>501</v>
       </c>
       <c r="B215" t="n">
-        <v>0</v>
+        <v>4950.369843695064</v>
       </c>
       <c r="C215" t="n">
-        <v>0</v>
+        <v>13653.58536367629</v>
       </c>
     </row>
     <row r="216">
@@ -2793,10 +2793,10 @@
         <v>502</v>
       </c>
       <c r="B216" t="n">
-        <v>2140.480629651258</v>
+        <v>6176.01611427562</v>
       </c>
       <c r="C216" t="n">
-        <v>5903.646781757358</v>
+        <v>17034.0329886869</v>
       </c>
     </row>
     <row r="217">
@@ -2804,10 +2804,10 @@
         <v>503</v>
       </c>
       <c r="B217" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C217" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="218">
@@ -2815,10 +2815,10 @@
         <v>504</v>
       </c>
       <c r="B218" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C218" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="219">
@@ -2826,10 +2826,10 @@
         <v>505</v>
       </c>
       <c r="B219" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C219" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="220">
@@ -2837,10 +2837,10 @@
         <v>506</v>
       </c>
       <c r="B220" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C220" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="221">
@@ -2848,10 +2848,10 @@
         <v>507</v>
       </c>
       <c r="B221" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C221" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="222">
@@ -2859,10 +2859,10 @@
         <v>508</v>
       </c>
       <c r="B222" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C222" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="223">
@@ -2870,10 +2870,10 @@
         <v>509</v>
       </c>
       <c r="B223" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C223" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="224">
@@ -2881,10 +2881,10 @@
         <v>510</v>
       </c>
       <c r="B224" t="n">
-        <v>6293.008293438715</v>
+        <v>10328.54377806308</v>
       </c>
       <c r="C224" t="n">
-        <v>17356.70841608356</v>
+        <v>28487.09462301311</v>
       </c>
     </row>
     <row r="225">
@@ -3046,10 +3046,10 @@
         <v>525</v>
       </c>
       <c r="B239" t="n">
-        <v>9686.003634797733</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C239" t="n">
-        <v>26714.90850911382</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="240">
@@ -3057,10 +3057,10 @@
         <v>526</v>
       </c>
       <c r="B240" t="n">
-        <v>10231.81959613874</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C240" t="n">
-        <v>28220.3202371927</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="241">
@@ -3068,10 +3068,10 @@
         <v>527</v>
       </c>
       <c r="B241" t="n">
-        <v>10649.67939851187</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C241" t="n">
-        <v>29372.8168509592</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="242">
@@ -3079,10 +3079,10 @@
         <v>528</v>
       </c>
       <c r="B242" t="n">
-        <v>8070.687362726562</v>
+        <v>10728.92339674058</v>
       </c>
       <c r="C242" t="n">
-        <v>22259.71439101196</v>
+        <v>29591.37924700981</v>
       </c>
     </row>
     <row r="243">
@@ -3090,10 +3090,10 @@
         <v>529</v>
       </c>
       <c r="B243" t="n">
-        <v>8167.710632158042</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C243" t="n">
-        <v>22527.3136882913</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="244">
@@ -3101,10 +3101,10 @@
         <v>530</v>
       </c>
       <c r="B244" t="n">
-        <v>8274.935142536411</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C244" t="n">
-        <v>22823.04896701882</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="245">
@@ -3112,10 +3112,10 @@
         <v>531</v>
       </c>
       <c r="B245" t="n">
-        <v>9996.023861394573</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C245" t="n">
-        <v>27569.9734359692</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="246">
@@ -3123,10 +3123,10 @@
         <v>532</v>
       </c>
       <c r="B246" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C246" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="247">
@@ -3134,10 +3134,10 @@
         <v>533</v>
       </c>
       <c r="B247" t="n">
-        <v>10672.37460599518</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C247" t="n">
-        <v>29435.41236654767</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="248">
@@ -3145,10 +3145,10 @@
         <v>534</v>
       </c>
       <c r="B248" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C248" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="249">
@@ -3189,10 +3189,10 @@
         <v>538</v>
       </c>
       <c r="B252" t="n">
-        <v>2666.633644515992</v>
+        <v>7137.715796175021</v>
       </c>
       <c r="C252" t="n">
-        <v>7354.82625513769</v>
+        <v>19686.49111113555</v>
       </c>
     </row>
     <row r="253">
@@ -3200,10 +3200,10 @@
         <v>539</v>
       </c>
       <c r="B253" t="n">
-        <v>0</v>
+        <v>3680.085914273101</v>
       </c>
       <c r="C253" t="n">
-        <v>0</v>
+        <v>10150.02287964115</v>
       </c>
     </row>
     <row r="254">
@@ -3211,10 +3211,10 @@
         <v>540</v>
       </c>
       <c r="B254" t="n">
-        <v>0</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C254" t="n">
-        <v>0</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="255">
@@ -3222,10 +3222,10 @@
         <v>541</v>
       </c>
       <c r="B255" t="n">
-        <v>0</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C255" t="n">
-        <v>0</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="256">
@@ -3233,10 +3233,10 @@
         <v>542</v>
       </c>
       <c r="B256" t="n">
-        <v>0</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C256" t="n">
-        <v>0</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="257">
@@ -3244,10 +3244,10 @@
         <v>543</v>
       </c>
       <c r="B257" t="n">
-        <v>0</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C257" t="n">
-        <v>0</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="258">
@@ -3255,10 +3255,10 @@
         <v>544</v>
       </c>
       <c r="B258" t="n">
-        <v>0</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C258" t="n">
-        <v>0</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="259">
@@ -3266,10 +3266,10 @@
         <v>545</v>
       </c>
       <c r="B259" t="n">
-        <v>2487.300163474301</v>
+        <v>6958.382315133329</v>
       </c>
       <c r="C259" t="n">
-        <v>6860.207657077488</v>
+        <v>19191.87251307534</v>
       </c>
     </row>
     <row r="260">
@@ -3277,10 +3277,10 @@
         <v>546</v>
       </c>
       <c r="B260" t="n">
-        <v>3901.193284849212</v>
+        <v>8372.27543650824</v>
       </c>
       <c r="C260" t="n">
-        <v>10759.8577917829</v>
+        <v>23091.52264778076</v>
       </c>
     </row>
     <row r="261">
@@ -3288,10 +3288,10 @@
         <v>547</v>
       </c>
       <c r="B261" t="n">
-        <v>5746.620025821905</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C261" t="n">
-        <v>15849.71821349924</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="262">
@@ -3299,10 +3299,10 @@
         <v>548</v>
       </c>
       <c r="B262" t="n">
-        <v>4342.898865330611</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C262" t="n">
-        <v>11978.12330307517</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="263">
@@ -3310,10 +3310,10 @@
         <v>549</v>
       </c>
       <c r="B263" t="n">
-        <v>5709.740530550902</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C263" t="n">
-        <v>15748.00109886926</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="264">
@@ -3321,10 +3321,10 @@
         <v>550</v>
       </c>
       <c r="B264" t="n">
-        <v>3913.606187237279</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C264" t="n">
-        <v>10794.09374338201</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="265">
@@ -3332,10 +3332,10 @@
         <v>551</v>
       </c>
       <c r="B265" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C265" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="266">
@@ -3343,10 +3343,10 @@
         <v>552</v>
       </c>
       <c r="B266" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C266" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="267">
@@ -3354,10 +3354,10 @@
         <v>553</v>
       </c>
       <c r="B267" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C267" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="268">
@@ -3365,10 +3365,10 @@
         <v>554</v>
       </c>
       <c r="B268" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C268" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="269">
@@ -3376,10 +3376,10 @@
         <v>555</v>
       </c>
       <c r="B269" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C269" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="270">
@@ -3387,10 +3387,10 @@
         <v>556</v>
       </c>
       <c r="B270" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C270" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="271">
@@ -3398,10 +3398,10 @@
         <v>557</v>
       </c>
       <c r="B271" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C271" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="272">
@@ -3409,10 +3409,10 @@
         <v>558</v>
       </c>
       <c r="B272" t="n">
-        <v>6997.352910028611</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C272" t="n">
-        <v>19299.35707703245</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="273">
@@ -3420,10 +3420,10 @@
         <v>559</v>
       </c>
       <c r="B273" t="n">
-        <v>0</v>
+        <v>9779.305357044783</v>
       </c>
       <c r="C273" t="n">
-        <v>0</v>
+        <v>26972.24342943307</v>
       </c>
     </row>
     <row r="274">
@@ -3431,10 +3431,10 @@
         <v>560</v>
       </c>
       <c r="B274" t="n">
-        <v>0</v>
+        <v>9996.65096565463</v>
       </c>
       <c r="C274" t="n">
-        <v>0</v>
+        <v>27571.70304846624</v>
       </c>
     </row>
     <row r="275">
@@ -3442,10 +3442,10 @@
         <v>561</v>
       </c>
       <c r="B275" t="n">
-        <v>1649.647793852841</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C275" t="n">
-        <v>4549.883682338757</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="276">
@@ -3453,10 +3453,10 @@
         <v>562</v>
       </c>
       <c r="B276" t="n">
-        <v>1649.647793852841</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C276" t="n">
-        <v>4549.883682338757</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="277">
@@ -3464,10 +3464,10 @@
         <v>563</v>
       </c>
       <c r="B277" t="n">
-        <v>0</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C277" t="n">
-        <v>0</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="278">
@@ -3475,10 +3475,10 @@
         <v>564</v>
       </c>
       <c r="B278" t="n">
-        <v>1649.647793852841</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C278" t="n">
-        <v>4549.883682338757</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="279">
@@ -3486,10 +3486,10 @@
         <v>565</v>
       </c>
       <c r="B279" t="n">
-        <v>10654.43087058984</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C279" t="n">
-        <v>29385.92185758862</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="280">
@@ -3497,10 +3497,10 @@
         <v>566</v>
       </c>
       <c r="B280" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C280" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="281">
@@ -3508,10 +3508,10 @@
         <v>567</v>
       </c>
       <c r="B281" t="n">
-        <v>0</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C281" t="n">
-        <v>0</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="282">
@@ -3519,10 +3519,10 @@
         <v>568</v>
       </c>
       <c r="B282" t="n">
-        <v>0</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C282" t="n">
-        <v>0</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="283">
@@ -3530,10 +3530,10 @@
         <v>569</v>
       </c>
       <c r="B283" t="n">
-        <v>0</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C283" t="n">
-        <v>0</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="284">
@@ -3541,10 +3541,10 @@
         <v>570</v>
       </c>
       <c r="B284" t="n">
-        <v>0</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C284" t="n">
-        <v>0</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="285">
@@ -3552,10 +3552,10 @@
         <v>571</v>
       </c>
       <c r="B285" t="n">
-        <v>1649.647793852841</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C285" t="n">
-        <v>4549.883682338757</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="286">
@@ -3563,10 +3563,10 @@
         <v>572</v>
       </c>
       <c r="B286" t="n">
-        <v>1649.647793852841</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C286" t="n">
-        <v>4549.883682338757</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="287">
@@ -3574,10 +3574,10 @@
         <v>573</v>
       </c>
       <c r="B287" t="n">
-        <v>1938.961669997816</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C287" t="n">
-        <v>5347.838548250955</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="288">
@@ -3585,10 +3585,10 @@
         <v>574</v>
       </c>
       <c r="B288" t="n">
-        <v>3913.606187237279</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C288" t="n">
-        <v>10794.09374338201</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="289">
@@ -3596,10 +3596,10 @@
         <v>575</v>
       </c>
       <c r="B289" t="n">
-        <v>4089.402655993988</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C289" t="n">
-        <v>11278.95692908108</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="290">
@@ -3607,10 +3607,10 @@
         <v>576</v>
       </c>
       <c r="B290" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C290" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="291">
@@ -3618,10 +3618,10 @@
         <v>577</v>
       </c>
       <c r="B291" t="n">
-        <v>6956.998276113732</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C291" t="n">
-        <v>19188.05520335963</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="292">
@@ -3629,10 +3629,10 @@
         <v>578</v>
       </c>
       <c r="B292" t="n">
-        <v>7025.505483901085</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C292" t="n">
-        <v>19377.00452211468</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="293">
@@ -3640,10 +3640,10 @@
         <v>579</v>
       </c>
       <c r="B293" t="n">
-        <v>0</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C293" t="n">
-        <v>0</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="294">
@@ -3651,10 +3651,10 @@
         <v>580</v>
       </c>
       <c r="B294" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C294" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="295">
@@ -3662,10 +3662,10 @@
         <v>581</v>
       </c>
       <c r="B295" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C295" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="296">
@@ -3673,10 +3673,10 @@
         <v>582</v>
       </c>
       <c r="B296" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C296" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="297">
@@ -3684,10 +3684,10 @@
         <v>583</v>
       </c>
       <c r="B297" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C297" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="298">
@@ -3695,10 +3695,10 @@
         <v>584</v>
       </c>
       <c r="B298" t="n">
-        <v>9583.095508839462</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C298" t="n">
-        <v>26431.07822435706</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="299">
@@ -3706,10 +3706,10 @@
         <v>585</v>
       </c>
       <c r="B299" t="n">
-        <v>7914.075982679272</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C299" t="n">
-        <v>21827.7654833718</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="300">
@@ -3717,10 +3717,10 @@
         <v>586</v>
       </c>
       <c r="B300" t="n">
-        <v>4306.182319570999</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C300" t="n">
-        <v>11876.85561851486</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="301">
@@ -3728,10 +3728,10 @@
         <v>587</v>
       </c>
       <c r="B301" t="n">
-        <v>2102.322267714388</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C301" t="n">
-        <v>5798.402432649447</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="302">
@@ -3739,10 +3739,10 @@
         <v>588</v>
       </c>
       <c r="B302" t="n">
-        <v>2748.333252112464</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C302" t="n">
-        <v>7580.161452651875</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="303">
@@ -3750,10 +3750,10 @@
         <v>589</v>
       </c>
       <c r="B303" t="n">
-        <v>1649.647793852841</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C303" t="n">
-        <v>4549.883682338757</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="304">
@@ -3761,10 +3761,10 @@
         <v>590</v>
       </c>
       <c r="B304" t="n">
-        <v>2650.593490323663</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C304" t="n">
-        <v>7310.586002100751</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="305">
@@ -3772,10 +3772,10 @@
         <v>591</v>
       </c>
       <c r="B305" t="n">
-        <v>4811.138560992982</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C305" t="n">
-        <v>13269.57239824338</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="306">
@@ -3783,10 +3783,10 @@
         <v>592</v>
       </c>
       <c r="B306" t="n">
-        <v>5880.356316974166</v>
+        <v>10351.43846863319</v>
       </c>
       <c r="C306" t="n">
-        <v>16218.57547570855</v>
+        <v>28550.2403317064</v>
       </c>
     </row>
     <row r="307">
@@ -3838,10 +3838,10 @@
         <v>597</v>
       </c>
       <c r="B311" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C311" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="312">
@@ -3849,10 +3849,10 @@
         <v>598</v>
       </c>
       <c r="B312" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C312" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="313">
@@ -3860,10 +3860,10 @@
         <v>599</v>
       </c>
       <c r="B313" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C313" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="314">
@@ -3871,10 +3871,10 @@
         <v>600</v>
       </c>
       <c r="B314" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C314" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="315">
@@ -3882,10 +3882,10 @@
         <v>601</v>
       </c>
       <c r="B315" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C315" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="316">
@@ -3893,10 +3893,10 @@
         <v>602</v>
       </c>
       <c r="B316" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C316" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="317">
@@ -3904,10 +3904,10 @@
         <v>603</v>
       </c>
       <c r="B317" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C317" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="318">
@@ -3915,10 +3915,10 @@
         <v>604</v>
       </c>
       <c r="B318" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C318" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="319">
@@ -3926,10 +3926,10 @@
         <v>605</v>
       </c>
       <c r="B319" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C319" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="320">
@@ -3937,10 +3937,10 @@
         <v>606</v>
       </c>
       <c r="B320" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C320" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="321">
@@ -3948,10 +3948,10 @@
         <v>607</v>
       </c>
       <c r="B321" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C321" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="322">
@@ -3959,10 +3959,10 @@
         <v>608</v>
       </c>
       <c r="B322" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C322" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="323">
@@ -3970,10 +3970,10 @@
         <v>609</v>
       </c>
       <c r="B323" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C323" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="324">
@@ -3981,10 +3981,10 @@
         <v>610</v>
       </c>
       <c r="B324" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C324" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="325">
@@ -3992,10 +3992,10 @@
         <v>611</v>
       </c>
       <c r="B325" t="n">
-        <v>8978.88728521926</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C325" t="n">
-        <v>24764.61514803953</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="326">
@@ -4003,10 +4003,10 @@
         <v>612</v>
       </c>
       <c r="B326" t="n">
-        <v>6442.740912541312</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C326" t="n">
-        <v>17769.68505443472</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="327">
@@ -4014,10 +4014,10 @@
         <v>613</v>
       </c>
       <c r="B327" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C327" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="328">
@@ -4025,10 +4025,10 @@
         <v>614</v>
       </c>
       <c r="B328" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C328" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="329">
@@ -4036,10 +4036,10 @@
         <v>615</v>
       </c>
       <c r="B329" t="n">
-        <v>5221.288087981926</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C329" t="n">
-        <v>14400.80334773442</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="330">
@@ -4047,10 +4047,10 @@
         <v>616</v>
       </c>
       <c r="B330" t="n">
-        <v>4202.236440499842</v>
+        <v>9167.688534285411</v>
       </c>
       <c r="C330" t="n">
-        <v>11590.16311312397</v>
+        <v>25285.34674028138</v>
       </c>
     </row>
     <row r="331">
@@ -4058,10 +4058,10 @@
         <v>617</v>
       </c>
       <c r="B331" t="n">
-        <v>0</v>
+        <v>9975.68237012327</v>
       </c>
       <c r="C331" t="n">
-        <v>0</v>
+        <v>27513.86969094277</v>
       </c>
     </row>
     <row r="332">
@@ -4069,10 +4069,10 @@
         <v>618</v>
       </c>
       <c r="B332" t="n">
-        <v>1649.647793852738</v>
+        <v>9966.717478079683</v>
       </c>
       <c r="C332" t="n">
-        <v>4549.883682338474</v>
+        <v>27489.14367598671</v>
       </c>
     </row>
     <row r="333">
@@ -4080,10 +4080,10 @@
         <v>619</v>
       </c>
       <c r="B333" t="n">
-        <v>6795.685774307415</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C333" t="n">
-        <v>18743.14016000264</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="334">
@@ -4091,10 +4091,10 @@
         <v>620</v>
       </c>
       <c r="B334" t="n">
-        <v>8032.944710977689</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C334" t="n">
-        <v>22155.6166096793</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="335">
@@ -4102,10 +4102,10 @@
         <v>621</v>
       </c>
       <c r="B335" t="n">
-        <v>9618.476955091568</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C335" t="n">
-        <v>26528.66357897632</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="336">
@@ -4113,10 +4113,10 @@
         <v>622</v>
       </c>
       <c r="B336" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C336" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="337">
@@ -4124,10 +4124,10 @@
         <v>623</v>
       </c>
       <c r="B337" t="n">
-        <v>10997.65195901894</v>
+        <v>10816.53264289492</v>
       </c>
       <c r="C337" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
   </sheetData>
@@ -4166,10 +4166,10 @@
         <v>5160</v>
       </c>
       <c r="B2" t="n">
-        <v>2104.096865820094</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>7563.756914925292</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -4177,10 +4177,10 @@
         <v>5161</v>
       </c>
       <c r="B3" t="n">
-        <v>1605.307122677738</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>5770.719517230988</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -4188,10 +4188,10 @@
         <v>5162</v>
       </c>
       <c r="B4" t="n">
-        <v>1512.48805673732</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>5437.055766645957</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -4199,10 +4199,10 @@
         <v>5163</v>
       </c>
       <c r="B5" t="n">
-        <v>3358.454019954424</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>12072.88990803568</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -4210,10 +4210,10 @@
         <v>5164</v>
       </c>
       <c r="B6" t="n">
-        <v>3699.457645448454</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>13298.72155687461</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -4221,10 +4221,10 @@
         <v>5165</v>
       </c>
       <c r="B7" t="n">
-        <v>4519.393840387589</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>16246.20851197313</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -4375,10 +4375,10 @@
         <v>5179</v>
       </c>
       <c r="B21" t="n">
-        <v>4486.089307824661</v>
+        <v>0</v>
       </c>
       <c r="C21" t="n">
-        <v>16126.4861776247</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -4386,10 +4386,10 @@
         <v>5180</v>
       </c>
       <c r="B22" t="n">
-        <v>4606.276735769084</v>
+        <v>0</v>
       </c>
       <c r="C22" t="n">
-        <v>16558.53305910104</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -4397,10 +4397,10 @@
         <v>5181</v>
       </c>
       <c r="B23" t="n">
-        <v>4266.134100467688</v>
+        <v>0</v>
       </c>
       <c r="C23" t="n">
-        <v>15335.79647714283</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -4408,10 +4408,10 @@
         <v>5182</v>
       </c>
       <c r="B24" t="n">
-        <v>3757.906203318487</v>
+        <v>3757.906203318435</v>
       </c>
       <c r="C24" t="n">
-        <v>13508.83102994041</v>
+        <v>13508.83102994023</v>
       </c>
     </row>
     <row r="25">
@@ -4419,10 +4419,10 @@
         <v>5183</v>
       </c>
       <c r="B25" t="n">
-        <v>2955.930541755406</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C25" t="n">
-        <v>10625.90816916933</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="26">
@@ -4430,10 +4430,10 @@
         <v>5184</v>
       </c>
       <c r="B26" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C26" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="27">
@@ -4441,10 +4441,10 @@
         <v>5185</v>
       </c>
       <c r="B27" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C27" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="28">
@@ -4452,10 +4452,10 @@
         <v>5186</v>
       </c>
       <c r="B28" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C28" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="29">
@@ -4463,10 +4463,10 @@
         <v>5187</v>
       </c>
       <c r="B29" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C29" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="30">
@@ -4474,10 +4474,10 @@
         <v>5188</v>
       </c>
       <c r="B30" t="n">
-        <v>3699.457645448506</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C30" t="n">
-        <v>13298.7215568748</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="31">
@@ -4518,10 +4518,10 @@
         <v>5192</v>
       </c>
       <c r="B34" t="n">
-        <v>5492.033204206517</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C34" t="n">
-        <v>19742.62915368468</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="35">
@@ -4529,10 +4529,10 @@
         <v>5193</v>
       </c>
       <c r="B35" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C35" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="36">
@@ -4540,10 +4540,10 @@
         <v>5194</v>
       </c>
       <c r="B36" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C36" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="37">
@@ -4551,10 +4551,10 @@
         <v>5195</v>
       </c>
       <c r="B37" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C37" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="38">
@@ -4562,10 +4562,10 @@
         <v>5196</v>
       </c>
       <c r="B38" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C38" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="39">
@@ -4573,10 +4573,10 @@
         <v>5197</v>
       </c>
       <c r="B39" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C39" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="40">
@@ -4584,10 +4584,10 @@
         <v>5198</v>
       </c>
       <c r="B40" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C40" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="41">
@@ -4595,10 +4595,10 @@
         <v>5199</v>
       </c>
       <c r="B41" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C41" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="42">
@@ -4606,10 +4606,10 @@
         <v>5200</v>
       </c>
       <c r="B42" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C42" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="43">
@@ -4617,10 +4617,10 @@
         <v>5201</v>
       </c>
       <c r="B43" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C43" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="44">
@@ -4628,10 +4628,10 @@
         <v>5202</v>
       </c>
       <c r="B44" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C44" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="45">
@@ -4639,10 +4639,10 @@
         <v>5203</v>
       </c>
       <c r="B45" t="n">
-        <v>4486.089307824611</v>
+        <v>0</v>
       </c>
       <c r="C45" t="n">
-        <v>16126.48617762452</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -4683,10 +4683,10 @@
         <v>5207</v>
       </c>
       <c r="B49" t="n">
-        <v>6440.735782742589</v>
+        <v>0</v>
       </c>
       <c r="C49" t="n">
-        <v>23153.00241414427</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -4694,10 +4694,10 @@
         <v>5208</v>
       </c>
       <c r="B50" t="n">
-        <v>7871.815531435896</v>
+        <v>0</v>
       </c>
       <c r="C50" t="n">
-        <v>28297.413548833</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -4705,10 +4705,10 @@
         <v>5209</v>
       </c>
       <c r="B51" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C51" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="52">
@@ -4716,10 +4716,10 @@
         <v>5210</v>
       </c>
       <c r="B52" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C52" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="53">
@@ -4727,10 +4727,10 @@
         <v>5211</v>
       </c>
       <c r="B53" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C53" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="54">
@@ -4738,10 +4738,10 @@
         <v>5212</v>
       </c>
       <c r="B54" t="n">
-        <v>8180.260414725609</v>
+        <v>8180.260414725616</v>
       </c>
       <c r="C54" t="n">
-        <v>29406.20381260566</v>
+        <v>29406.20381260569</v>
       </c>
     </row>
     <row r="55">
@@ -4793,10 +4793,10 @@
         <v>5217</v>
       </c>
       <c r="B59" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C59" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="60">
@@ -4804,10 +4804,10 @@
         <v>5218</v>
       </c>
       <c r="B60" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C60" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="61">
@@ -4815,10 +4815,10 @@
         <v>5219</v>
       </c>
       <c r="B61" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C61" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="62">
@@ -4826,10 +4826,10 @@
         <v>5220</v>
       </c>
       <c r="B62" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C62" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="63">
@@ -4837,10 +4837,10 @@
         <v>5221</v>
       </c>
       <c r="B63" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C63" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="64">
@@ -4848,10 +4848,10 @@
         <v>5222</v>
       </c>
       <c r="B64" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C64" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="65">
@@ -4859,10 +4859,10 @@
         <v>5223</v>
       </c>
       <c r="B65" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C65" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="66">
@@ -4870,10 +4870,10 @@
         <v>5224</v>
       </c>
       <c r="B66" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C66" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="67">
@@ -4881,10 +4881,10 @@
         <v>5225</v>
       </c>
       <c r="B67" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C67" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="68">
@@ -4991,10 +4991,10 @@
         <v>5235</v>
       </c>
       <c r="B77" t="n">
-        <v>7873.231468214149</v>
+        <v>0</v>
       </c>
       <c r="C77" t="n">
-        <v>28302.50352438098</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78">
@@ -5002,10 +5002,10 @@
         <v>5236</v>
       </c>
       <c r="B78" t="n">
-        <v>8180.260414725557</v>
+        <v>0</v>
       </c>
       <c r="C78" t="n">
-        <v>29406.20381260548</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -5013,10 +5013,10 @@
         <v>5237</v>
       </c>
       <c r="B79" t="n">
-        <v>8437.954933007895</v>
+        <v>0</v>
       </c>
       <c r="C79" t="n">
-        <v>30332.55788225838</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
@@ -5233,10 +5233,10 @@
         <v>5257</v>
       </c>
       <c r="B99" t="n">
-        <v>1605.307122677687</v>
+        <v>0</v>
       </c>
       <c r="C99" t="n">
-        <v>5770.719517230804</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100">
@@ -5244,10 +5244,10 @@
         <v>5258</v>
       </c>
       <c r="B100" t="n">
-        <v>1512.488056737244</v>
+        <v>0</v>
       </c>
       <c r="C100" t="n">
-        <v>5437.055766645681</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101">
@@ -5255,10 +5255,10 @@
         <v>5259</v>
       </c>
       <c r="B101" t="n">
-        <v>1528.632894778551</v>
+        <v>0</v>
       </c>
       <c r="C101" t="n">
-        <v>5495.092842960461</v>
+        <v>0</v>
       </c>
     </row>
     <row r="102">
@@ -5266,10 +5266,10 @@
         <v>5260</v>
       </c>
       <c r="B102" t="n">
-        <v>1845.333289930335</v>
+        <v>0</v>
       </c>
       <c r="C102" t="n">
-        <v>6633.559822642609</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -5574,10 +5574,10 @@
         <v>5288</v>
       </c>
       <c r="B130" t="n">
-        <v>5181.365160847776</v>
+        <v>0</v>
       </c>
       <c r="C130" t="n">
-        <v>18625.84712745172</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131">
@@ -5684,10 +5684,10 @@
         <v>5298</v>
       </c>
       <c r="B140" t="n">
-        <v>6217.958231119063</v>
+        <v>0</v>
       </c>
       <c r="C140" t="n">
-        <v>22352.16701822926</v>
+        <v>0</v>
       </c>
     </row>
     <row r="141">
@@ -5750,10 +5750,10 @@
         <v>5304</v>
       </c>
       <c r="B146" t="n">
-        <v>6005.178953988655</v>
+        <v>0</v>
       </c>
       <c r="C146" t="n">
-        <v>21587.27317950352</v>
+        <v>0</v>
       </c>
     </row>
     <row r="147">
@@ -5761,10 +5761,10 @@
         <v>5305</v>
       </c>
       <c r="B147" t="n">
-        <v>8004.922191931879</v>
+        <v>0</v>
       </c>
       <c r="C147" t="n">
-        <v>28775.90217742411</v>
+        <v>0</v>
       </c>
     </row>
     <row r="148">
@@ -5783,10 +5783,10 @@
         <v>5307</v>
       </c>
       <c r="B149" t="n">
-        <v>7954.247763642288</v>
+        <v>0</v>
       </c>
       <c r="C149" t="n">
-        <v>28593.73895879497</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150">
@@ -5794,10 +5794,10 @@
         <v>5308</v>
       </c>
       <c r="B150" t="n">
-        <v>8022.344547721922</v>
+        <v>0</v>
       </c>
       <c r="C150" t="n">
-        <v>28838.53164388162</v>
+        <v>0</v>
       </c>
     </row>
     <row r="151">
@@ -5827,10 +5827,10 @@
         <v>5311</v>
       </c>
       <c r="B153" t="n">
-        <v>3045.80832514813</v>
+        <v>0</v>
       </c>
       <c r="C153" t="n">
-        <v>10948.99866784269</v>
+        <v>0</v>
       </c>
     </row>
     <row r="154">
@@ -6036,10 +6036,10 @@
         <v>5330</v>
       </c>
       <c r="B172" t="n">
-        <v>5423.07054654082</v>
+        <v>0</v>
       </c>
       <c r="C172" t="n">
-        <v>19494.72384701182</v>
+        <v>0</v>
       </c>
     </row>
     <row r="173">
@@ -6047,10 +6047,10 @@
         <v>5331</v>
       </c>
       <c r="B173" t="n">
-        <v>5538.003146077993</v>
+        <v>0</v>
       </c>
       <c r="C173" t="n">
-        <v>19907.88079744566</v>
+        <v>0</v>
       </c>
     </row>
     <row r="174">
@@ -6289,10 +6289,10 @@
         <v>5353</v>
       </c>
       <c r="B195" t="n">
-        <v>1605.307122677656</v>
+        <v>0</v>
       </c>
       <c r="C195" t="n">
-        <v>5770.719517230693</v>
+        <v>0</v>
       </c>
     </row>
     <row r="196">
@@ -6300,10 +6300,10 @@
         <v>5354</v>
       </c>
       <c r="B196" t="n">
-        <v>1512.48805673732</v>
+        <v>0</v>
       </c>
       <c r="C196" t="n">
-        <v>5437.055766645957</v>
+        <v>0</v>
       </c>
     </row>
     <row r="197">
@@ -6311,10 +6311,10 @@
         <v>5355</v>
       </c>
       <c r="B197" t="n">
-        <v>1528.632894778576</v>
+        <v>0</v>
       </c>
       <c r="C197" t="n">
-        <v>5495.092842960549</v>
+        <v>0</v>
       </c>
     </row>
     <row r="198">
@@ -6322,10 +6322,10 @@
         <v>5356</v>
       </c>
       <c r="B198" t="n">
-        <v>1845.333289930281</v>
+        <v>0</v>
       </c>
       <c r="C198" t="n">
-        <v>6633.559822642414</v>
+        <v>0</v>
       </c>
     </row>
     <row r="199">
@@ -6553,10 +6553,10 @@
         <v>5377</v>
       </c>
       <c r="B219" t="n">
-        <v>1605.307122677698</v>
+        <v>0</v>
       </c>
       <c r="C219" t="n">
-        <v>5770.719517230842</v>
+        <v>0</v>
       </c>
     </row>
     <row r="220">
@@ -6564,10 +6564,10 @@
         <v>5378</v>
       </c>
       <c r="B220" t="n">
-        <v>1512.488056737244</v>
+        <v>0</v>
       </c>
       <c r="C220" t="n">
-        <v>5437.055766645681</v>
+        <v>0</v>
       </c>
     </row>
     <row r="221">
@@ -6575,10 +6575,10 @@
         <v>5379</v>
       </c>
       <c r="B221" t="n">
-        <v>1528.632894778632</v>
+        <v>0</v>
       </c>
       <c r="C221" t="n">
-        <v>5495.092842960752</v>
+        <v>0</v>
       </c>
     </row>
     <row r="222">
@@ -6586,10 +6586,10 @@
         <v>5380</v>
       </c>
       <c r="B222" t="n">
-        <v>1845.333289930281</v>
+        <v>0</v>
       </c>
       <c r="C222" t="n">
-        <v>6633.559822642414</v>
+        <v>0</v>
       </c>
     </row>
     <row r="223">
@@ -7070,10 +7070,10 @@
         <v>5424</v>
       </c>
       <c r="B266" t="n">
-        <v>2104.096865820102</v>
+        <v>0</v>
       </c>
       <c r="C266" t="n">
-        <v>7563.756914925321</v>
+        <v>0</v>
       </c>
     </row>
     <row r="267">
@@ -7081,10 +7081,10 @@
         <v>5425</v>
       </c>
       <c r="B267" t="n">
-        <v>1605.30712267771</v>
+        <v>0</v>
       </c>
       <c r="C267" t="n">
-        <v>5770.719517230886</v>
+        <v>0</v>
       </c>
     </row>
     <row r="268">
@@ -7334,10 +7334,10 @@
         <v>5448</v>
       </c>
       <c r="B290" t="n">
-        <v>2298.04108081247</v>
+        <v>0</v>
       </c>
       <c r="C290" t="n">
-        <v>8260.942924318728</v>
+        <v>0</v>
       </c>
     </row>
     <row r="291">
@@ -7345,10 +7345,10 @@
         <v>5449</v>
       </c>
       <c r="B291" t="n">
-        <v>1690.60284730891</v>
+        <v>0</v>
       </c>
       <c r="C291" t="n">
-        <v>6077.338541037733</v>
+        <v>0</v>
       </c>
     </row>
     <row r="292">
@@ -7356,10 +7356,10 @@
         <v>5450</v>
       </c>
       <c r="B292" t="n">
-        <v>1566.603360959052</v>
+        <v>0</v>
       </c>
       <c r="C292" t="n">
-        <v>5631.588163494937</v>
+        <v>0</v>
       </c>
     </row>
     <row r="293">
@@ -7367,10 +7367,10 @@
         <v>5451</v>
       </c>
       <c r="B293" t="n">
-        <v>1392.403727304189</v>
+        <v>0</v>
       </c>
       <c r="C293" t="n">
-        <v>5005.379501223644</v>
+        <v>0</v>
       </c>
     </row>
     <row r="294">
@@ -7378,10 +7378,10 @@
         <v>5452</v>
       </c>
       <c r="B294" t="n">
-        <v>1516.479755457432</v>
+        <v>0</v>
       </c>
       <c r="C294" t="n">
-        <v>5451.405029404246</v>
+        <v>0</v>
       </c>
     </row>
     <row r="295">
@@ -7389,10 +7389,10 @@
         <v>5453</v>
       </c>
       <c r="B295" t="n">
-        <v>1899.108708620582</v>
+        <v>0</v>
       </c>
       <c r="C295" t="n">
-        <v>6826.870407140262</v>
+        <v>0</v>
       </c>
     </row>
     <row r="296">
@@ -7422,10 +7422,10 @@
         <v>5456</v>
       </c>
       <c r="B298" t="n">
-        <v>5181.365160847776</v>
+        <v>0</v>
       </c>
       <c r="C298" t="n">
-        <v>18625.84712745172</v>
+        <v>0</v>
       </c>
     </row>
     <row r="299">
@@ -7433,10 +7433,10 @@
         <v>5457</v>
       </c>
       <c r="B299" t="n">
-        <v>5887.19176508303</v>
+        <v>0</v>
       </c>
       <c r="C299" t="n">
-        <v>21163.13566451811</v>
+        <v>0</v>
       </c>
     </row>
     <row r="300">
@@ -7444,10 +7444,10 @@
         <v>5458</v>
       </c>
       <c r="B300" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C300" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="301">
@@ -7455,10 +7455,10 @@
         <v>5459</v>
       </c>
       <c r="B301" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C301" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="302">
@@ -7521,10 +7521,10 @@
         <v>5465</v>
       </c>
       <c r="B307" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C307" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="308">
@@ -7532,10 +7532,10 @@
         <v>5466</v>
       </c>
       <c r="B308" t="n">
-        <v>6217.958231119064</v>
+        <v>0</v>
       </c>
       <c r="C308" t="n">
-        <v>22352.16701822926</v>
+        <v>0</v>
       </c>
     </row>
     <row r="309">
@@ -7675,10 +7675,10 @@
         <v>5479</v>
       </c>
       <c r="B321" t="n">
-        <v>4739.905750759392</v>
+        <v>0</v>
       </c>
       <c r="C321" t="n">
-        <v>17038.89943509184</v>
+        <v>0</v>
       </c>
     </row>
     <row r="322">
@@ -7686,10 +7686,10 @@
         <v>5480</v>
       </c>
       <c r="B322" t="n">
-        <v>4660.746443195231</v>
+        <v>0</v>
       </c>
       <c r="C322" t="n">
-        <v>16754.33945608358</v>
+        <v>0</v>
       </c>
     </row>
     <row r="323">
@@ -7697,10 +7697,10 @@
         <v>5481</v>
       </c>
       <c r="B323" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C323" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="324">
@@ -7708,10 +7708,10 @@
         <v>5482</v>
       </c>
       <c r="B324" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C324" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="325">
@@ -7719,10 +7719,10 @@
         <v>5483</v>
       </c>
       <c r="B325" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C325" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="326">
@@ -7730,10 +7730,10 @@
         <v>5484</v>
       </c>
       <c r="B326" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C326" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="327">
@@ -7741,10 +7741,10 @@
         <v>5485</v>
       </c>
       <c r="B327" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C327" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="328">
@@ -7752,10 +7752,10 @@
         <v>5486</v>
       </c>
       <c r="B328" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C328" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="329">
@@ -7763,10 +7763,10 @@
         <v>5487</v>
       </c>
       <c r="B329" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C329" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="330">
@@ -7774,10 +7774,10 @@
         <v>5488</v>
       </c>
       <c r="B330" t="n">
-        <v>8437.954933007895</v>
+        <v>8298.991031199892</v>
       </c>
       <c r="C330" t="n">
-        <v>30332.55788225838</v>
+        <v>29833.01378317262</v>
       </c>
     </row>
     <row r="331">
@@ -7785,10 +7785,10 @@
         <v>5489</v>
       </c>
       <c r="B331" t="n">
-        <v>3384.8070443907</v>
+        <v>0</v>
       </c>
       <c r="C331" t="n">
-        <v>12167.62312780662</v>
+        <v>0</v>
       </c>
     </row>
     <row r="332">

</xml_diff>

<commit_message>
LSHP and Chiller max bound up to  70MW
</commit_message>
<xml_diff>
--- a/first_stage_optimization/lshp_operation.xlsx
+++ b/first_stage_optimization/lshp_operation.xlsx
@@ -439,10 +439,10 @@
         <v>288</v>
       </c>
       <c r="B2" t="n">
-        <v>14661.83753471311</v>
+        <v>11197.08202174817</v>
       </c>
       <c r="C2" t="n">
-        <v>40438.72613346702</v>
+        <v>30882.6047416915</v>
       </c>
     </row>
     <row r="3">
@@ -450,10 +450,10 @@
         <v>289</v>
       </c>
       <c r="B3" t="n">
-        <v>16227.52394141103</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C3" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="4">
@@ -461,10 +461,10 @@
         <v>290</v>
       </c>
       <c r="B4" t="n">
-        <v>16227.52394141103</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C4" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="5">
@@ -472,10 +472,10 @@
         <v>291</v>
       </c>
       <c r="B5" t="n">
-        <v>16227.52394141103</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C5" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="6">
@@ -483,10 +483,10 @@
         <v>292</v>
       </c>
       <c r="B6" t="n">
-        <v>16227.52394141103</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C6" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="7">
@@ -494,10 +494,10 @@
         <v>293</v>
       </c>
       <c r="B7" t="n">
-        <v>16227.52394141103</v>
+        <v>15640.50738895312</v>
       </c>
       <c r="C7" t="n">
-        <v>44757.0364176621</v>
+        <v>43137.98958642726</v>
       </c>
     </row>
     <row r="8">
@@ -505,10 +505,10 @@
         <v>294</v>
       </c>
       <c r="B8" t="n">
-        <v>16227.52394141103</v>
+        <v>15771.71513208502</v>
       </c>
       <c r="C8" t="n">
-        <v>44757.0364176621</v>
+        <v>43499.8728755129</v>
       </c>
     </row>
     <row r="9">
@@ -538,10 +538,10 @@
         <v>297</v>
       </c>
       <c r="B11" t="n">
-        <v>10892.0487091489</v>
+        <v>7427.29319618396</v>
       </c>
       <c r="C11" t="n">
-        <v>30041.29419241133</v>
+        <v>20485.1728006358</v>
       </c>
     </row>
     <row r="12">
@@ -549,10 +549,10 @@
         <v>298</v>
       </c>
       <c r="B12" t="n">
-        <v>13613.69344088266</v>
+        <v>2671.138940993995</v>
       </c>
       <c r="C12" t="n">
-        <v>37547.84619713782</v>
+        <v>7367.252286321891</v>
       </c>
     </row>
     <row r="13">
@@ -571,10 +571,10 @@
         <v>300</v>
       </c>
       <c r="B14" t="n">
-        <v>16227.52394141103</v>
+        <v>11725.51941396181</v>
       </c>
       <c r="C14" t="n">
-        <v>44757.0364176621</v>
+        <v>32340.08474253159</v>
       </c>
     </row>
     <row r="15">
@@ -582,10 +582,10 @@
         <v>301</v>
       </c>
       <c r="B15" t="n">
-        <v>16227.52394141103</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C15" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="16">
@@ -593,10 +593,10 @@
         <v>302</v>
       </c>
       <c r="B16" t="n">
-        <v>16227.52394141103</v>
+        <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>44757.0364176621</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -648,10 +648,10 @@
         <v>307</v>
       </c>
       <c r="B21" t="n">
-        <v>5628.311937815829</v>
+        <v>2420.200107322064</v>
       </c>
       <c r="C21" t="n">
-        <v>15523.41338581821</v>
+        <v>6675.139394804341</v>
       </c>
     </row>
     <row r="22">
@@ -659,10 +659,10 @@
         <v>308</v>
       </c>
       <c r="B22" t="n">
-        <v>6906.990958459112</v>
+        <v>3442.235445494172</v>
       </c>
       <c r="C22" t="n">
-        <v>19050.13032058033</v>
+        <v>9494.008928804804</v>
       </c>
     </row>
     <row r="23">
@@ -670,10 +670,10 @@
         <v>309</v>
       </c>
       <c r="B23" t="n">
-        <v>11687.76275546055</v>
+        <v>8223.007242495609</v>
       </c>
       <c r="C23" t="n">
-        <v>32235.9483292592</v>
+        <v>22679.82693748368</v>
       </c>
     </row>
     <row r="24">
@@ -681,10 +681,10 @@
         <v>310</v>
       </c>
       <c r="B24" t="n">
-        <v>16227.52394141103</v>
+        <v>12332.30114269007</v>
       </c>
       <c r="C24" t="n">
-        <v>44757.0364176621</v>
+        <v>34013.64578784662</v>
       </c>
     </row>
     <row r="25">
@@ -692,10 +692,10 @@
         <v>311</v>
       </c>
       <c r="B25" t="n">
-        <v>16227.52394141103</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C25" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="26">
@@ -703,10 +703,10 @@
         <v>312</v>
       </c>
       <c r="B26" t="n">
-        <v>16227.52394141103</v>
+        <v>14184.39603300014</v>
       </c>
       <c r="C26" t="n">
-        <v>44757.0364176621</v>
+        <v>39121.8975922415</v>
       </c>
     </row>
     <row r="27">
@@ -714,10 +714,10 @@
         <v>313</v>
       </c>
       <c r="B27" t="n">
-        <v>16227.52394141103</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C27" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="28">
@@ -725,10 +725,10 @@
         <v>314</v>
       </c>
       <c r="B28" t="n">
-        <v>16227.52394141103</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C28" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="29">
@@ -736,10 +736,10 @@
         <v>315</v>
       </c>
       <c r="B29" t="n">
-        <v>16227.52394141103</v>
+        <v>15700.36452466098</v>
       </c>
       <c r="C29" t="n">
-        <v>44757.0364176621</v>
+        <v>43303.08119328029</v>
       </c>
     </row>
     <row r="30">
@@ -747,10 +747,10 @@
         <v>316</v>
       </c>
       <c r="B30" t="n">
-        <v>16227.52394141103</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C30" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="31">
@@ -758,10 +758,10 @@
         <v>317</v>
       </c>
       <c r="B31" t="n">
-        <v>16227.52394141103</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C31" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="32">
@@ -769,10 +769,10 @@
         <v>318</v>
       </c>
       <c r="B32" t="n">
-        <v>16227.52394141103</v>
+        <v>15771.71513208502</v>
       </c>
       <c r="C32" t="n">
-        <v>44757.0364176621</v>
+        <v>43499.8728755129</v>
       </c>
     </row>
     <row r="33">
@@ -780,10 +780,10 @@
         <v>319</v>
       </c>
       <c r="B33" t="n">
-        <v>16227.52394141103</v>
+        <v>4574.87140815473</v>
       </c>
       <c r="C33" t="n">
-        <v>44757.0364176621</v>
+        <v>12617.92538160311</v>
       </c>
     </row>
     <row r="34">
@@ -802,10 +802,10 @@
         <v>321</v>
       </c>
       <c r="B35" t="n">
-        <v>10892.0487091489</v>
+        <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>30041.29419241133</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -813,10 +813,10 @@
         <v>322</v>
       </c>
       <c r="B36" t="n">
-        <v>8570.769153159979</v>
+        <v>5106.013640195039</v>
       </c>
       <c r="C36" t="n">
-        <v>23638.98697671562</v>
+        <v>14082.8655849401</v>
       </c>
     </row>
     <row r="37">
@@ -824,10 +824,10 @@
         <v>323</v>
       </c>
       <c r="B37" t="n">
-        <v>16227.52394141103</v>
+        <v>2420.200107322064</v>
       </c>
       <c r="C37" t="n">
-        <v>44757.0364176621</v>
+        <v>6675.139394804341</v>
       </c>
     </row>
     <row r="38">
@@ -934,10 +934,10 @@
         <v>333</v>
       </c>
       <c r="B47" t="n">
-        <v>9011.154174682662</v>
+        <v>5546.398661717728</v>
       </c>
       <c r="C47" t="n">
-        <v>24853.6102622672</v>
+        <v>15297.4888704917</v>
       </c>
     </row>
     <row r="48">
@@ -945,10 +945,10 @@
         <v>334</v>
       </c>
       <c r="B48" t="n">
-        <v>15797.05665565501</v>
+        <v>12332.30114269007</v>
       </c>
       <c r="C48" t="n">
-        <v>43569.76717962214</v>
+        <v>34013.64578784662</v>
       </c>
     </row>
     <row r="49">
@@ -956,10 +956,10 @@
         <v>335</v>
       </c>
       <c r="B49" t="n">
-        <v>16227.52394141103</v>
+        <v>13180.5251643192</v>
       </c>
       <c r="C49" t="n">
-        <v>44757.0364176621</v>
+        <v>36353.12737255779</v>
       </c>
     </row>
     <row r="50">
@@ -967,10 +967,10 @@
         <v>336</v>
       </c>
       <c r="B50" t="n">
-        <v>16227.52394141103</v>
+        <v>11197.08202174817</v>
       </c>
       <c r="C50" t="n">
-        <v>44757.0364176621</v>
+        <v>30882.6047416915</v>
       </c>
     </row>
     <row r="51">
@@ -978,10 +978,10 @@
         <v>337</v>
       </c>
       <c r="B51" t="n">
-        <v>16227.52394141103</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C51" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="52">
@@ -989,10 +989,10 @@
         <v>338</v>
       </c>
       <c r="B52" t="n">
-        <v>15400.42560310273</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C52" t="n">
-        <v>42475.82145336401</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="53">
@@ -1000,10 +1000,10 @@
         <v>339</v>
       </c>
       <c r="B53" t="n">
-        <v>16227.52394141103</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C53" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="54">
@@ -1011,10 +1011,10 @@
         <v>340</v>
       </c>
       <c r="B54" t="n">
-        <v>15967.42976796647</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C54" t="n">
-        <v>44039.67223844971</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="55">
@@ -1022,10 +1022,10 @@
         <v>341</v>
       </c>
       <c r="B55" t="n">
-        <v>16079.27149234439</v>
+        <v>13873.55516262652</v>
       </c>
       <c r="C55" t="n">
-        <v>44348.14222740612</v>
+        <v>38264.56925270922</v>
       </c>
     </row>
     <row r="56">
@@ -1033,10 +1033,10 @@
         <v>342</v>
       </c>
       <c r="B56" t="n">
-        <v>13356.16694275438</v>
+        <v>9891.411429789443</v>
       </c>
       <c r="C56" t="n">
-        <v>36837.56390780921</v>
+        <v>27281.44251603368</v>
       </c>
     </row>
     <row r="57">
@@ -1231,10 +1231,10 @@
         <v>360</v>
       </c>
       <c r="B74" t="n">
-        <v>3622.480496173405</v>
+        <v>0</v>
       </c>
       <c r="C74" t="n">
-        <v>9991.14172161289</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -1242,10 +1242,10 @@
         <v>361</v>
       </c>
       <c r="B75" t="n">
-        <v>3851.506422101356</v>
+        <v>2420.200107322062</v>
       </c>
       <c r="C75" t="n">
-        <v>10622.81675375922</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="76">
@@ -1253,10 +1253,10 @@
         <v>362</v>
       </c>
       <c r="B76" t="n">
-        <v>4117.917007473863</v>
+        <v>2420.200107322062</v>
       </c>
       <c r="C76" t="n">
-        <v>11357.60219081162</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="77">
@@ -1264,10 +1264,10 @@
         <v>363</v>
       </c>
       <c r="B77" t="n">
-        <v>16227.52394141103</v>
+        <v>2420.200107322064</v>
       </c>
       <c r="C77" t="n">
-        <v>44757.0364176621</v>
+        <v>6675.139394804341</v>
       </c>
     </row>
     <row r="78">
@@ -1275,10 +1275,10 @@
         <v>364</v>
       </c>
       <c r="B78" t="n">
-        <v>13113.2559399548</v>
+        <v>0</v>
       </c>
       <c r="C78" t="n">
-        <v>36167.5925284537</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -1286,10 +1286,10 @@
         <v>365</v>
       </c>
       <c r="B79" t="n">
-        <v>4994.891653253849</v>
+        <v>2420.200107322062</v>
       </c>
       <c r="C79" t="n">
-        <v>13776.38069948952</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="80">
@@ -1297,10 +1297,10 @@
         <v>366</v>
       </c>
       <c r="B80" t="n">
-        <v>5468.613123466752</v>
+        <v>2420.200107322062</v>
       </c>
       <c r="C80" t="n">
-        <v>15082.94904415491</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="81">
@@ -1495,10 +1495,10 @@
         <v>384</v>
       </c>
       <c r="B98" t="n">
-        <v>6183.793196442298</v>
+        <v>2719.037683477357</v>
       </c>
       <c r="C98" t="n">
-        <v>17055.48291234832</v>
+        <v>7499.361520572798</v>
       </c>
     </row>
     <row r="99">
@@ -1506,10 +1506,10 @@
         <v>385</v>
       </c>
       <c r="B99" t="n">
-        <v>16227.52394141103</v>
+        <v>2990.384331759942</v>
       </c>
       <c r="C99" t="n">
-        <v>44757.0364176621</v>
+        <v>8247.761083121106</v>
       </c>
     </row>
     <row r="100">
@@ -1517,10 +1517,10 @@
         <v>386</v>
       </c>
       <c r="B100" t="n">
-        <v>16227.52394141103</v>
+        <v>3268.251465062969</v>
       </c>
       <c r="C100" t="n">
-        <v>44757.0364176621</v>
+        <v>9014.144756281385</v>
       </c>
     </row>
     <row r="101">
@@ -1528,10 +1528,10 @@
         <v>387</v>
       </c>
       <c r="B101" t="n">
-        <v>16227.52394141103</v>
+        <v>6948.505853923947</v>
       </c>
       <c r="C101" t="n">
-        <v>44757.0364176621</v>
+        <v>19164.63230467252</v>
       </c>
     </row>
     <row r="102">
@@ -1539,10 +1539,10 @@
         <v>388</v>
       </c>
       <c r="B102" t="n">
-        <v>16227.52394141103</v>
+        <v>2420.200107322062</v>
       </c>
       <c r="C102" t="n">
-        <v>44757.0364176621</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="103">
@@ -1550,10 +1550,10 @@
         <v>389</v>
       </c>
       <c r="B103" t="n">
-        <v>4994.891653253849</v>
+        <v>2420.200107322062</v>
       </c>
       <c r="C103" t="n">
-        <v>13776.38069948952</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="104">
@@ -1561,10 +1561,10 @@
         <v>390</v>
       </c>
       <c r="B104" t="n">
-        <v>7952.96607559232</v>
+        <v>4488.21056262738</v>
       </c>
       <c r="C104" t="n">
-        <v>21935.02801529472</v>
+        <v>12378.9066235192</v>
       </c>
     </row>
     <row r="105">
@@ -1726,10 +1726,10 @@
         <v>405</v>
       </c>
       <c r="B119" t="n">
-        <v>4018.932957836866</v>
+        <v>2420.200107322062</v>
       </c>
       <c r="C119" t="n">
-        <v>11084.59487741211</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="120">
@@ -1737,10 +1737,10 @@
         <v>406</v>
       </c>
       <c r="B120" t="n">
-        <v>7538.776746350087</v>
+        <v>4074.021233385152</v>
       </c>
       <c r="C120" t="n">
-        <v>20792.65491144769</v>
+        <v>11236.53351967219</v>
       </c>
     </row>
     <row r="121">
@@ -1748,10 +1748,10 @@
         <v>407</v>
       </c>
       <c r="B121" t="n">
-        <v>8152.132178745583</v>
+        <v>4687.376665780643</v>
       </c>
       <c r="C121" t="n">
-        <v>22484.34684940512</v>
+        <v>12928.2254576296</v>
       </c>
     </row>
     <row r="122">
@@ -1759,10 +1759,10 @@
         <v>408</v>
       </c>
       <c r="B122" t="n">
-        <v>10086.38505501611</v>
+        <v>6621.629542051171</v>
       </c>
       <c r="C122" t="n">
-        <v>27819.19810192959</v>
+        <v>18263.07671015408</v>
       </c>
     </row>
     <row r="123">
@@ -1770,10 +1770,10 @@
         <v>409</v>
       </c>
       <c r="B123" t="n">
-        <v>10284.60671765093</v>
+        <v>6819.851204685992</v>
       </c>
       <c r="C123" t="n">
-        <v>28365.91208031273</v>
+        <v>18809.79068853721</v>
       </c>
     </row>
     <row r="124">
@@ -1781,10 +1781,10 @@
         <v>410</v>
       </c>
       <c r="B124" t="n">
-        <v>16227.52394141103</v>
+        <v>7099.280057115846</v>
       </c>
       <c r="C124" t="n">
-        <v>44757.0364176621</v>
+        <v>19580.48172985087</v>
       </c>
     </row>
     <row r="125">
@@ -1792,10 +1792,10 @@
         <v>411</v>
       </c>
       <c r="B125" t="n">
-        <v>16227.52394141103</v>
+        <v>7496.823652848921</v>
       </c>
       <c r="C125" t="n">
-        <v>44757.0364176621</v>
+        <v>20676.94433598069</v>
       </c>
     </row>
     <row r="126">
@@ -1803,10 +1803,10 @@
         <v>412</v>
       </c>
       <c r="B126" t="n">
-        <v>8089.609984129404</v>
+        <v>5654.012943367195</v>
       </c>
       <c r="C126" t="n">
-        <v>22311.90475956741</v>
+        <v>15594.2991750234</v>
       </c>
     </row>
     <row r="127">
@@ -1814,10 +1814,10 @@
         <v>413</v>
       </c>
       <c r="B127" t="n">
-        <v>16227.52394141103</v>
+        <v>4015.178821929269</v>
       </c>
       <c r="C127" t="n">
-        <v>44757.0364176621</v>
+        <v>11074.24061769019</v>
       </c>
     </row>
     <row r="128">
@@ -1825,10 +1825,10 @@
         <v>414</v>
       </c>
       <c r="B128" t="n">
-        <v>6535.69842051366</v>
+        <v>3070.942907548726</v>
       </c>
       <c r="C128" t="n">
-        <v>18026.0705994282</v>
+        <v>8469.949207652695</v>
       </c>
     </row>
     <row r="129">
@@ -1836,10 +1836,10 @@
         <v>415</v>
       </c>
       <c r="B129" t="n">
-        <v>6150.872376992415</v>
+        <v>2686.116864027475</v>
       </c>
       <c r="C129" t="n">
-        <v>16964.68419774852</v>
+        <v>7408.562805972993</v>
       </c>
     </row>
     <row r="130">
@@ -1847,10 +1847,10 @@
         <v>416</v>
       </c>
       <c r="B130" t="n">
-        <v>6038.775086831522</v>
+        <v>2574.019573866587</v>
       </c>
       <c r="C130" t="n">
-        <v>16655.5093343395</v>
+        <v>7099.38794256399</v>
       </c>
     </row>
     <row r="131">
@@ -1858,10 +1858,10 @@
         <v>417</v>
       </c>
       <c r="B131" t="n">
-        <v>5855.842708277934</v>
+        <v>2420.200107322064</v>
       </c>
       <c r="C131" t="n">
-        <v>16150.96463864512</v>
+        <v>6675.139394804341</v>
       </c>
     </row>
     <row r="132">
@@ -1869,10 +1869,10 @@
         <v>418</v>
       </c>
       <c r="B132" t="n">
-        <v>4200.058406524801</v>
+        <v>0</v>
       </c>
       <c r="C132" t="n">
-        <v>11584.15589068562</v>
+        <v>0</v>
       </c>
     </row>
     <row r="133">
@@ -1979,10 +1979,10 @@
         <v>428</v>
       </c>
       <c r="B142" t="n">
-        <v>5349.056572928629</v>
+        <v>2420.200107322062</v>
       </c>
       <c r="C142" t="n">
-        <v>14753.20083945501</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="143">
@@ -1990,10 +1990,10 @@
         <v>429</v>
       </c>
       <c r="B143" t="n">
-        <v>6072.162767063096</v>
+        <v>2607.407254098156</v>
       </c>
       <c r="C143" t="n">
-        <v>16747.59569486012</v>
+        <v>7191.4743030846</v>
       </c>
     </row>
     <row r="144">
@@ -2001,10 +2001,10 @@
         <v>430</v>
       </c>
       <c r="B144" t="n">
-        <v>7392.41216357169</v>
+        <v>3927.656650606756</v>
       </c>
       <c r="C144" t="n">
-        <v>20388.9676338741</v>
+        <v>10832.84624209859</v>
       </c>
     </row>
     <row r="145">
@@ -2012,10 +2012,10 @@
         <v>431</v>
       </c>
       <c r="B145" t="n">
-        <v>8541.22723488989</v>
+        <v>5076.471721924955</v>
       </c>
       <c r="C145" t="n">
-        <v>23557.5075891864</v>
+        <v>14001.38619741089</v>
       </c>
     </row>
     <row r="146">
@@ -2023,10 +2023,10 @@
         <v>432</v>
       </c>
       <c r="B146" t="n">
-        <v>10291.95742004125</v>
+        <v>6827.201907076305</v>
       </c>
       <c r="C146" t="n">
-        <v>28386.18600847124</v>
+        <v>18830.06461669572</v>
       </c>
     </row>
     <row r="147">
@@ -2034,10 +2034,10 @@
         <v>433</v>
       </c>
       <c r="B147" t="n">
-        <v>11026.63922527536</v>
+        <v>7561.883712310421</v>
       </c>
       <c r="C147" t="n">
-        <v>30412.50748739662</v>
+        <v>20856.3860956211</v>
       </c>
     </row>
     <row r="148">
@@ -2045,10 +2045,10 @@
         <v>434</v>
       </c>
       <c r="B148" t="n">
-        <v>11475.17202671491</v>
+        <v>7829.974092509725</v>
       </c>
       <c r="C148" t="n">
-        <v>31649.60311585024</v>
+        <v>21595.80456470652</v>
       </c>
     </row>
     <row r="149">
@@ -2056,10 +2056,10 @@
         <v>435</v>
       </c>
       <c r="B149" t="n">
-        <v>11447.5183340251</v>
+        <v>7982.762821060161</v>
       </c>
       <c r="C149" t="n">
-        <v>31573.33163196463</v>
+        <v>22017.2102401891</v>
       </c>
     </row>
     <row r="150">
@@ -2067,10 +2067,10 @@
         <v>436</v>
       </c>
       <c r="B150" t="n">
-        <v>16227.52394141103</v>
+        <v>7680.581968994567</v>
       </c>
       <c r="C150" t="n">
-        <v>44757.0364176621</v>
+        <v>21183.7670451921</v>
       </c>
     </row>
     <row r="151">
@@ -2078,10 +2078,10 @@
         <v>437</v>
       </c>
       <c r="B151" t="n">
-        <v>13245.85570408344</v>
+        <v>9781.100191118503</v>
       </c>
       <c r="C151" t="n">
-        <v>36533.31514229832</v>
+        <v>26977.1937505228</v>
       </c>
     </row>
     <row r="152">
@@ -2089,10 +2089,10 @@
         <v>438</v>
       </c>
       <c r="B152" t="n">
-        <v>16227.52394141103</v>
+        <v>5809.303108874029</v>
       </c>
       <c r="C152" t="n">
-        <v>44757.0364176621</v>
+        <v>16022.60404876681</v>
       </c>
     </row>
     <row r="153">
@@ -2100,10 +2100,10 @@
         <v>439</v>
       </c>
       <c r="B153" t="n">
-        <v>8903.385898554039</v>
+        <v>5438.630385589105</v>
       </c>
       <c r="C153" t="n">
-        <v>24556.3752264865</v>
+        <v>15000.25383471099</v>
       </c>
     </row>
     <row r="154">
@@ -2111,10 +2111,10 @@
         <v>440</v>
       </c>
       <c r="B154" t="n">
-        <v>8782.912519094494</v>
+        <v>5318.157006129553</v>
       </c>
       <c r="C154" t="n">
-        <v>24224.09832143941</v>
+        <v>14667.97692966388</v>
       </c>
     </row>
     <row r="155">
@@ -2122,10 +2122,10 @@
         <v>441</v>
       </c>
       <c r="B155" t="n">
-        <v>6895.755311556394</v>
+        <v>3430.999798591454</v>
       </c>
       <c r="C155" t="n">
-        <v>19019.14135027182</v>
+        <v>9463.019958496297</v>
       </c>
     </row>
     <row r="156">
@@ -2133,10 +2133,10 @@
         <v>442</v>
       </c>
       <c r="B156" t="n">
-        <v>5736.285052507169</v>
+        <v>2420.200107322064</v>
       </c>
       <c r="C156" t="n">
-        <v>15821.21338560971</v>
+        <v>6675.139394804341</v>
       </c>
     </row>
     <row r="157">
@@ -2155,10 +2155,10 @@
         <v>444</v>
       </c>
       <c r="B158" t="n">
-        <v>16227.52394141103</v>
+        <v>7731.830712880651</v>
       </c>
       <c r="C158" t="n">
-        <v>44757.0364176621</v>
+        <v>21325.11589821185</v>
       </c>
     </row>
     <row r="159">
@@ -2166,10 +2166,10 @@
         <v>445</v>
       </c>
       <c r="B159" t="n">
-        <v>16227.52394141103</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C159" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="160">
@@ -2177,10 +2177,10 @@
         <v>446</v>
       </c>
       <c r="B160" t="n">
-        <v>16227.52394141103</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C160" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="161">
@@ -2265,10 +2265,10 @@
         <v>454</v>
       </c>
       <c r="B168" t="n">
-        <v>5546.557472199574</v>
+        <v>2420.200107322064</v>
       </c>
       <c r="C168" t="n">
-        <v>15297.92688472881</v>
+        <v>6675.139394804341</v>
       </c>
     </row>
     <row r="169">
@@ -2276,10 +2276,10 @@
         <v>455</v>
       </c>
       <c r="B169" t="n">
-        <v>6253.125660203575</v>
+        <v>2788.370147238635</v>
       </c>
       <c r="C169" t="n">
-        <v>17246.70836465352</v>
+        <v>7690.586972877994</v>
       </c>
     </row>
     <row r="170">
@@ -2287,10 +2287,10 @@
         <v>456</v>
       </c>
       <c r="B170" t="n">
-        <v>6183.793196442298</v>
+        <v>2719.037683477357</v>
       </c>
       <c r="C170" t="n">
-        <v>17055.48291234832</v>
+        <v>7499.361520572798</v>
       </c>
     </row>
     <row r="171">
@@ -2298,10 +2298,10 @@
         <v>457</v>
       </c>
       <c r="B171" t="n">
-        <v>6455.139844724877</v>
+        <v>2990.384331759942</v>
       </c>
       <c r="C171" t="n">
-        <v>17803.88247489661</v>
+        <v>8247.761083121106</v>
       </c>
     </row>
     <row r="172">
@@ -2309,10 +2309,10 @@
         <v>458</v>
       </c>
       <c r="B172" t="n">
-        <v>16227.52394141103</v>
+        <v>3268.251465062969</v>
       </c>
       <c r="C172" t="n">
-        <v>44757.0364176621</v>
+        <v>9014.144756281385</v>
       </c>
     </row>
     <row r="173">
@@ -2320,10 +2320,10 @@
         <v>459</v>
       </c>
       <c r="B173" t="n">
-        <v>16227.52394141103</v>
+        <v>3800.567685719266</v>
       </c>
       <c r="C173" t="n">
-        <v>44757.0364176621</v>
+        <v>10482.32293057619</v>
       </c>
     </row>
     <row r="174">
@@ -2331,10 +2331,10 @@
         <v>460</v>
       </c>
       <c r="B174" t="n">
-        <v>12942.558574349</v>
+        <v>9477.803061384062</v>
       </c>
       <c r="C174" t="n">
-        <v>35696.79314856054</v>
+        <v>26140.67175678501</v>
       </c>
     </row>
     <row r="175">
@@ -2342,10 +2342,10 @@
         <v>461</v>
       </c>
       <c r="B175" t="n">
-        <v>13075.26811572656</v>
+        <v>9610.512602761624</v>
       </c>
       <c r="C175" t="n">
-        <v>36062.81853837674</v>
+        <v>26506.69714660122</v>
       </c>
     </row>
     <row r="176">
@@ -2353,10 +2353,10 @@
         <v>462</v>
       </c>
       <c r="B176" t="n">
-        <v>13356.16694275438</v>
+        <v>9891.411429789443</v>
       </c>
       <c r="C176" t="n">
-        <v>36837.56390780921</v>
+        <v>27281.44251603368</v>
       </c>
     </row>
     <row r="177">
@@ -2529,10 +2529,10 @@
         <v>478</v>
       </c>
       <c r="B192" t="n">
-        <v>5072.773245545554</v>
+        <v>0</v>
       </c>
       <c r="C192" t="n">
-        <v>13991.18545189972</v>
+        <v>0</v>
       </c>
     </row>
     <row r="193">
@@ -2540,10 +2540,10 @@
         <v>479</v>
       </c>
       <c r="B193" t="n">
-        <v>5559.296919778698</v>
+        <v>2420.200107322064</v>
       </c>
       <c r="C193" t="n">
-        <v>15333.06347866011</v>
+        <v>6675.139394804341</v>
       </c>
     </row>
     <row r="194">
@@ -2551,10 +2551,10 @@
         <v>480</v>
       </c>
       <c r="B194" t="n">
-        <v>6183.793196442298</v>
+        <v>2719.037683477357</v>
       </c>
       <c r="C194" t="n">
-        <v>17055.48291234832</v>
+        <v>7499.361520572798</v>
       </c>
     </row>
     <row r="195">
@@ -2562,10 +2562,10 @@
         <v>481</v>
       </c>
       <c r="B195" t="n">
-        <v>16227.52394141103</v>
+        <v>2990.384331759942</v>
       </c>
       <c r="C195" t="n">
-        <v>44757.0364176621</v>
+        <v>8247.761083121106</v>
       </c>
     </row>
     <row r="196">
@@ -2573,10 +2573,10 @@
         <v>482</v>
       </c>
       <c r="B196" t="n">
-        <v>16227.52394141103</v>
+        <v>3268.251465062969</v>
       </c>
       <c r="C196" t="n">
-        <v>44757.0364176621</v>
+        <v>9014.144756281385</v>
       </c>
     </row>
     <row r="197">
@@ -2584,10 +2584,10 @@
         <v>483</v>
       </c>
       <c r="B197" t="n">
-        <v>16227.52394141103</v>
+        <v>3800.567685719266</v>
       </c>
       <c r="C197" t="n">
-        <v>44757.0364176621</v>
+        <v>10482.32293057619</v>
       </c>
     </row>
     <row r="198">
@@ -2595,10 +2595,10 @@
         <v>484</v>
       </c>
       <c r="B198" t="n">
-        <v>16227.52394141103</v>
+        <v>6512.570198329713</v>
       </c>
       <c r="C198" t="n">
-        <v>44757.0364176621</v>
+        <v>17962.28078859199</v>
       </c>
     </row>
     <row r="199">
@@ -2606,10 +2606,10 @@
         <v>485</v>
       </c>
       <c r="B199" t="n">
-        <v>16227.52394141103</v>
+        <v>6706.333521350718</v>
       </c>
       <c r="C199" t="n">
-        <v>44757.0364176621</v>
+        <v>18496.69824723629</v>
       </c>
     </row>
     <row r="200">
@@ -2617,10 +2617,10 @@
         <v>486</v>
       </c>
       <c r="B200" t="n">
-        <v>10507.18058270959</v>
+        <v>7042.425069744652</v>
       </c>
       <c r="C200" t="n">
-        <v>28979.79172208783</v>
+        <v>19423.67033031231</v>
       </c>
     </row>
     <row r="201">
@@ -2782,10 +2782,10 @@
         <v>501</v>
       </c>
       <c r="B215" t="n">
-        <v>4018.932957836866</v>
+        <v>2420.200107322062</v>
       </c>
       <c r="C215" t="n">
-        <v>11084.59487741211</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="216">
@@ -2793,10 +2793,10 @@
         <v>502</v>
       </c>
       <c r="B216" t="n">
-        <v>5072.773245545554</v>
+        <v>0</v>
       </c>
       <c r="C216" t="n">
-        <v>13991.18545189972</v>
+        <v>0</v>
       </c>
     </row>
     <row r="217">
@@ -2804,10 +2804,10 @@
         <v>503</v>
       </c>
       <c r="B217" t="n">
-        <v>5559.296919778698</v>
+        <v>2420.200107322064</v>
       </c>
       <c r="C217" t="n">
-        <v>15333.06347866011</v>
+        <v>6675.139394804341</v>
       </c>
     </row>
     <row r="218">
@@ -2815,10 +2815,10 @@
         <v>504</v>
       </c>
       <c r="B218" t="n">
-        <v>6183.793196442298</v>
+        <v>2719.037683477357</v>
       </c>
       <c r="C218" t="n">
-        <v>17055.48291234832</v>
+        <v>7499.361520572798</v>
       </c>
     </row>
     <row r="219">
@@ -2826,10 +2826,10 @@
         <v>505</v>
       </c>
       <c r="B219" t="n">
-        <v>6455.139844724877</v>
+        <v>2990.384331759942</v>
       </c>
       <c r="C219" t="n">
-        <v>17803.88247489661</v>
+        <v>8247.761083121106</v>
       </c>
     </row>
     <row r="220">
@@ -2837,10 +2837,10 @@
         <v>506</v>
       </c>
       <c r="B220" t="n">
-        <v>16227.52394141103</v>
+        <v>5970.788395873496</v>
       </c>
       <c r="C220" t="n">
-        <v>44757.0364176621</v>
+        <v>16467.99564992831</v>
       </c>
     </row>
     <row r="221">
@@ -2848,10 +2848,10 @@
         <v>507</v>
       </c>
       <c r="B221" t="n">
-        <v>9945.630804522254</v>
+        <v>6480.875291557313</v>
       </c>
       <c r="C221" t="n">
-        <v>27430.984648168</v>
+        <v>17874.86325639248</v>
       </c>
     </row>
     <row r="222">
@@ -2859,10 +2859,10 @@
         <v>508</v>
       </c>
       <c r="B222" t="n">
-        <v>16227.52394141103</v>
+        <v>6512.570198329713</v>
       </c>
       <c r="C222" t="n">
-        <v>44757.0364176621</v>
+        <v>17962.28078859199</v>
       </c>
     </row>
     <row r="223">
@@ -2870,10 +2870,10 @@
         <v>509</v>
       </c>
       <c r="B223" t="n">
-        <v>10171.08903431566</v>
+        <v>6706.333521350718</v>
       </c>
       <c r="C223" t="n">
-        <v>28052.81963901181</v>
+        <v>18496.69824723629</v>
       </c>
     </row>
     <row r="224">
@@ -2881,10 +2881,10 @@
         <v>510</v>
       </c>
       <c r="B224" t="n">
-        <v>7952.96607559232</v>
+        <v>4488.21056262738</v>
       </c>
       <c r="C224" t="n">
-        <v>21935.02801529472</v>
+        <v>12378.9066235192</v>
       </c>
     </row>
     <row r="225">
@@ -4003,10 +4003,10 @@
         <v>612</v>
       </c>
       <c r="B326" t="n">
-        <v>16227.52394141103</v>
+        <v>0</v>
       </c>
       <c r="C326" t="n">
-        <v>44757.0364176621</v>
+        <v>0</v>
       </c>
     </row>
     <row r="327">
@@ -4014,10 +4014,10 @@
         <v>613</v>
       </c>
       <c r="B327" t="n">
-        <v>16227.52394141103</v>
+        <v>2420.200107322064</v>
       </c>
       <c r="C327" t="n">
-        <v>44757.0364176621</v>
+        <v>6675.139394804341</v>
       </c>
     </row>
     <row r="328">
@@ -4298,10 +4298,10 @@
         <v>5172</v>
       </c>
       <c r="B14" t="n">
-        <v>5309.422455413364</v>
+        <v>7563.007057174681</v>
       </c>
       <c r="C14" t="n">
-        <v>19086.18441658103</v>
+        <v>27187.31625696217</v>
       </c>
     </row>
     <row r="15">
@@ -4408,10 +4408,10 @@
         <v>5182</v>
       </c>
       <c r="B24" t="n">
-        <v>1874.820568382635</v>
+        <v>1874.820568382665</v>
       </c>
       <c r="C24" t="n">
-        <v>6739.559983528256</v>
+        <v>6739.55998352836</v>
       </c>
     </row>
     <row r="25">
@@ -4419,10 +4419,10 @@
         <v>5183</v>
       </c>
       <c r="B25" t="n">
-        <v>2686.906972228544</v>
+        <v>1856.899955603442</v>
       </c>
       <c r="C25" t="n">
-        <v>9658.828697999836</v>
+        <v>6675.139394804318</v>
       </c>
     </row>
     <row r="26">
@@ -4441,10 +4441,10 @@
         <v>5185</v>
       </c>
       <c r="B27" t="n">
-        <v>0</v>
+        <v>2284.204171165625</v>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>8211.202333606079</v>
       </c>
     </row>
     <row r="28">
@@ -4452,10 +4452,10 @@
         <v>5186</v>
       </c>
       <c r="B28" t="n">
-        <v>12450.57728705825</v>
+        <v>12379.33303735631</v>
       </c>
       <c r="C28" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="29">
@@ -4463,10 +4463,10 @@
         <v>5187</v>
       </c>
       <c r="B29" t="n">
-        <v>0</v>
+        <v>2299.850630719266</v>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>8267.447850894478</v>
       </c>
     </row>
     <row r="30">
@@ -4474,10 +4474,10 @@
         <v>5188</v>
       </c>
       <c r="B30" t="n">
-        <v>0</v>
+        <v>9272.421191446763</v>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>33332.27716090422</v>
       </c>
     </row>
     <row r="31">
@@ -4485,10 +4485,10 @@
         <v>5189</v>
       </c>
       <c r="B31" t="n">
-        <v>0</v>
+        <v>1856.899955603447</v>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="32">
@@ -4496,10 +4496,10 @@
         <v>5190</v>
       </c>
       <c r="B32" t="n">
-        <v>2070.628765404916</v>
+        <v>2070.628765404943</v>
       </c>
       <c r="C32" t="n">
-        <v>7443.446590787222</v>
+        <v>7443.44659078732</v>
       </c>
     </row>
     <row r="33">
@@ -4650,10 +4650,10 @@
         <v>5204</v>
       </c>
       <c r="B46" t="n">
-        <v>0</v>
+        <v>2346.064435599156</v>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>8433.57612754539</v>
       </c>
     </row>
     <row r="47">
@@ -4661,10 +4661,10 @@
         <v>5205</v>
       </c>
       <c r="B47" t="n">
-        <v>2157.297466391308</v>
+        <v>2157.297466391335</v>
       </c>
       <c r="C47" t="n">
-        <v>7755.00115704428</v>
+        <v>7755.001157044377</v>
       </c>
     </row>
     <row r="48">
@@ -4672,10 +4672,10 @@
         <v>5206</v>
       </c>
       <c r="B48" t="n">
-        <v>1874.820568382635</v>
+        <v>1874.820568382665</v>
       </c>
       <c r="C48" t="n">
-        <v>6739.559983528256</v>
+        <v>6739.55998352836</v>
       </c>
     </row>
     <row r="49">
@@ -4683,10 +4683,10 @@
         <v>5207</v>
       </c>
       <c r="B49" t="n">
-        <v>12450.57728705825</v>
+        <v>12379.33303735631</v>
       </c>
       <c r="C49" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="50">
@@ -4694,10 +4694,10 @@
         <v>5208</v>
       </c>
       <c r="B50" t="n">
-        <v>0</v>
+        <v>2552.756939774566</v>
       </c>
       <c r="C50" t="n">
-        <v>0</v>
+        <v>9176.589380935055</v>
       </c>
     </row>
     <row r="51">
@@ -4705,10 +4705,10 @@
         <v>5209</v>
       </c>
       <c r="B51" t="n">
-        <v>0</v>
+        <v>2518.087048222285</v>
       </c>
       <c r="C51" t="n">
-        <v>0</v>
+        <v>9051.958886860313</v>
       </c>
     </row>
     <row r="52">
@@ -4738,10 +4738,10 @@
         <v>5212</v>
       </c>
       <c r="B54" t="n">
-        <v>12450.57728705825</v>
+        <v>12379.33303735631</v>
       </c>
       <c r="C54" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="55">
@@ -4749,10 +4749,10 @@
         <v>5213</v>
       </c>
       <c r="B55" t="n">
-        <v>0</v>
+        <v>1856.899955603447</v>
       </c>
       <c r="C55" t="n">
-        <v>0</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="56">
@@ -4793,10 +4793,10 @@
         <v>5217</v>
       </c>
       <c r="B59" t="n">
-        <v>0</v>
+        <v>1856.899955603447</v>
       </c>
       <c r="C59" t="n">
-        <v>0</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="60">
@@ -4804,10 +4804,10 @@
         <v>5218</v>
       </c>
       <c r="B60" t="n">
-        <v>0</v>
+        <v>2205.349870521857</v>
       </c>
       <c r="C60" t="n">
-        <v>0</v>
+        <v>7927.738786155077</v>
       </c>
     </row>
     <row r="61">
@@ -4815,10 +4815,10 @@
         <v>5219</v>
       </c>
       <c r="B61" t="n">
-        <v>2288.64786677666</v>
+        <v>2033.817988805349</v>
       </c>
       <c r="C61" t="n">
-        <v>8227.176423939933</v>
+        <v>7311.120094525737</v>
       </c>
     </row>
     <row r="62">
@@ -4903,10 +4903,10 @@
         <v>5227</v>
       </c>
       <c r="B69" t="n">
-        <v>0</v>
+        <v>2268.320949722101</v>
       </c>
       <c r="C69" t="n">
-        <v>0</v>
+        <v>8154.105710358214</v>
       </c>
     </row>
     <row r="70">
@@ -4914,10 +4914,10 @@
         <v>5228</v>
       </c>
       <c r="B70" t="n">
-        <v>0</v>
+        <v>2346.064435599156</v>
       </c>
       <c r="C70" t="n">
-        <v>0</v>
+        <v>8433.57612754539</v>
       </c>
     </row>
     <row r="71">
@@ -4925,10 +4925,10 @@
         <v>5229</v>
       </c>
       <c r="B71" t="n">
-        <v>0</v>
+        <v>2157.297466391335</v>
       </c>
       <c r="C71" t="n">
-        <v>0</v>
+        <v>7755.001157044377</v>
       </c>
     </row>
     <row r="72">
@@ -5002,10 +5002,10 @@
         <v>5236</v>
       </c>
       <c r="B78" t="n">
-        <v>0</v>
+        <v>8662.985600275406</v>
       </c>
       <c r="C78" t="n">
-        <v>0</v>
+        <v>31141.49272421562</v>
       </c>
     </row>
     <row r="79">
@@ -5057,10 +5057,10 @@
         <v>5241</v>
       </c>
       <c r="B83" t="n">
-        <v>12450.57728705825</v>
+        <v>12379.33303735631</v>
       </c>
       <c r="C83" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="84">
@@ -5211,10 +5211,10 @@
         <v>5255</v>
       </c>
       <c r="B97" t="n">
-        <v>1867.586593058722</v>
+        <v>0</v>
       </c>
       <c r="C97" t="n">
-        <v>6713.555462649259</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -5266,10 +5266,10 @@
         <v>5260</v>
       </c>
       <c r="B102" t="n">
-        <v>12388.0429580152</v>
+        <v>12379.33303735631</v>
       </c>
       <c r="C102" t="n">
-        <v>44532.23951244205</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="103">
@@ -5277,10 +5277,10 @@
         <v>5261</v>
       </c>
       <c r="B103" t="n">
-        <v>1867.586593058722</v>
+        <v>12379.33303735631</v>
       </c>
       <c r="C103" t="n">
-        <v>6713.555462649259</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="104">
@@ -5288,10 +5288,10 @@
         <v>5262</v>
       </c>
       <c r="B104" t="n">
-        <v>2070.628765404916</v>
+        <v>2070.628765404943</v>
       </c>
       <c r="C104" t="n">
-        <v>7443.446590787222</v>
+        <v>7443.44659078732</v>
       </c>
     </row>
     <row r="105">
@@ -5783,10 +5783,10 @@
         <v>5307</v>
       </c>
       <c r="B149" t="n">
-        <v>12450.57728705825</v>
+        <v>9800.278967776228</v>
       </c>
       <c r="C149" t="n">
-        <v>44757.0364176621</v>
+        <v>35229.80762666676</v>
       </c>
     </row>
     <row r="150">
@@ -5794,10 +5794,10 @@
         <v>5308</v>
       </c>
       <c r="B150" t="n">
-        <v>12450.57728705825</v>
+        <v>12379.33303735631</v>
       </c>
       <c r="C150" t="n">
-        <v>44757.03641766209</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="151">
@@ -5805,10 +5805,10 @@
         <v>5309</v>
       </c>
       <c r="B151" t="n">
-        <v>12450.57728705825</v>
+        <v>12379.33303735631</v>
       </c>
       <c r="C151" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="152">
@@ -6014,10 +6014,10 @@
         <v>5328</v>
       </c>
       <c r="B170" t="n">
-        <v>1867.586593058724</v>
+        <v>0</v>
       </c>
       <c r="C170" t="n">
-        <v>6713.555462649267</v>
+        <v>0</v>
       </c>
     </row>
     <row r="171">
@@ -6025,10 +6025,10 @@
         <v>5329</v>
       </c>
       <c r="B171" t="n">
-        <v>12450.57728705825</v>
+        <v>0</v>
       </c>
       <c r="C171" t="n">
-        <v>44757.0364176621</v>
+        <v>0</v>
       </c>
     </row>
     <row r="172">
@@ -6036,10 +6036,10 @@
         <v>5330</v>
       </c>
       <c r="B172" t="n">
-        <v>12450.57728705825</v>
+        <v>12379.33303735631</v>
       </c>
       <c r="C172" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="173">
@@ -6047,10 +6047,10 @@
         <v>5331</v>
       </c>
       <c r="B173" t="n">
-        <v>12450.57728705825</v>
+        <v>12379.33303735631</v>
       </c>
       <c r="C173" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869556</v>
       </c>
     </row>
     <row r="174">
@@ -6058,10 +6058,10 @@
         <v>5332</v>
       </c>
       <c r="B174" t="n">
-        <v>12450.57728705825</v>
+        <v>5422.989787194354</v>
       </c>
       <c r="C174" t="n">
-        <v>44757.0364176621</v>
+        <v>19494.43353525137</v>
       </c>
     </row>
     <row r="175">
@@ -6069,10 +6069,10 @@
         <v>5333</v>
       </c>
       <c r="B175" t="n">
-        <v>1867.586593058722</v>
+        <v>0</v>
       </c>
       <c r="C175" t="n">
-        <v>6713.555462649259</v>
+        <v>0</v>
       </c>
     </row>
     <row r="176">
@@ -6080,10 +6080,10 @@
         <v>5334</v>
       </c>
       <c r="B176" t="n">
-        <v>2070.628765404916</v>
+        <v>2070.628765404943</v>
       </c>
       <c r="C176" t="n">
-        <v>7443.446590787222</v>
+        <v>7443.44659078732</v>
       </c>
     </row>
     <row r="177">
@@ -6091,10 +6091,10 @@
         <v>5335</v>
       </c>
       <c r="B177" t="n">
-        <v>0</v>
+        <v>1856.899955603447</v>
       </c>
       <c r="C177" t="n">
-        <v>0</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="178">
@@ -6300,10 +6300,10 @@
         <v>5354</v>
       </c>
       <c r="B196" t="n">
-        <v>0</v>
+        <v>12379.33303735631</v>
       </c>
       <c r="C196" t="n">
-        <v>0</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="197">
@@ -6311,10 +6311,10 @@
         <v>5355</v>
       </c>
       <c r="B197" t="n">
-        <v>0</v>
+        <v>12379.33303735631</v>
       </c>
       <c r="C197" t="n">
-        <v>0</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="198">
@@ -6322,10 +6322,10 @@
         <v>5356</v>
       </c>
       <c r="B198" t="n">
-        <v>11521.83592488392</v>
+        <v>0</v>
       </c>
       <c r="C198" t="n">
-        <v>41418.4192587105</v>
+        <v>0</v>
       </c>
     </row>
     <row r="199">
@@ -7367,10 +7367,10 @@
         <v>5451</v>
       </c>
       <c r="B293" t="n">
-        <v>5818.181396072483</v>
+        <v>12379.33303735631</v>
       </c>
       <c r="C293" t="n">
-        <v>20915.05884624785</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="294">
@@ -7378,10 +7378,10 @@
         <v>5452</v>
       </c>
       <c r="B294" t="n">
-        <v>1867.586593058724</v>
+        <v>2364.6056215037</v>
       </c>
       <c r="C294" t="n">
-        <v>6713.555462649267</v>
+        <v>8500.227537646582</v>
       </c>
     </row>
     <row r="295">
@@ -7389,10 +7389,10 @@
         <v>5453</v>
       </c>
       <c r="B295" t="n">
-        <v>1867.586593058722</v>
+        <v>1856.899955603448</v>
       </c>
       <c r="C295" t="n">
-        <v>6713.555462649259</v>
+        <v>6675.139394804341</v>
       </c>
     </row>
     <row r="296">
@@ -7565,10 +7565,10 @@
         <v>5469</v>
       </c>
       <c r="B311" t="n">
-        <v>0</v>
+        <v>2327.1776631764</v>
       </c>
       <c r="C311" t="n">
-        <v>0</v>
+        <v>8365.682411322605</v>
       </c>
     </row>
     <row r="312">
@@ -7598,10 +7598,10 @@
         <v>5472</v>
       </c>
       <c r="B314" t="n">
-        <v>1867.586593058722</v>
+        <v>1856.899955603442</v>
       </c>
       <c r="C314" t="n">
-        <v>6713.555462649259</v>
+        <v>6675.139394804317</v>
       </c>
     </row>
     <row r="315">
@@ -7609,10 +7609,10 @@
         <v>5473</v>
       </c>
       <c r="B315" t="n">
-        <v>3866.5968391644</v>
+        <v>1856.899955603447</v>
       </c>
       <c r="C315" t="n">
-        <v>13899.54951910404</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="316">
@@ -7620,10 +7620,10 @@
         <v>5474</v>
       </c>
       <c r="B316" t="n">
-        <v>12450.57728705825</v>
+        <v>1856.899955603447</v>
       </c>
       <c r="C316" t="n">
-        <v>44757.0364176621</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="317">
@@ -7631,10 +7631,10 @@
         <v>5475</v>
       </c>
       <c r="B317" t="n">
-        <v>12450.57728705825</v>
+        <v>7707.830164704253</v>
       </c>
       <c r="C317" t="n">
-        <v>44757.0364176621</v>
+        <v>27707.92288815489</v>
       </c>
     </row>
     <row r="318">
@@ -7642,10 +7642,10 @@
         <v>5476</v>
       </c>
       <c r="B318" t="n">
-        <v>12450.57728705825</v>
+        <v>1856.89995560341</v>
       </c>
       <c r="C318" t="n">
-        <v>44757.0364176621</v>
+        <v>6675.139394804203</v>
       </c>
     </row>
     <row r="319">
@@ -7653,10 +7653,10 @@
         <v>5477</v>
       </c>
       <c r="B319" t="n">
-        <v>1867.586593058724</v>
+        <v>0</v>
       </c>
       <c r="C319" t="n">
-        <v>6713.555462649267</v>
+        <v>0</v>
       </c>
     </row>
     <row r="320">
@@ -7664,10 +7664,10 @@
         <v>5478</v>
       </c>
       <c r="B320" t="n">
-        <v>1867.586593058722</v>
+        <v>1856.89995560344</v>
       </c>
       <c r="C320" t="n">
-        <v>6713.555462649259</v>
+        <v>6675.13939480431</v>
       </c>
     </row>
     <row r="321">
@@ -7675,10 +7675,10 @@
         <v>5479</v>
       </c>
       <c r="B321" t="n">
-        <v>12450.57728705825</v>
+        <v>12379.33303735631</v>
       </c>
       <c r="C321" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="322">
@@ -7686,10 +7686,10 @@
         <v>5480</v>
       </c>
       <c r="B322" t="n">
-        <v>12450.57728705825</v>
+        <v>12379.33303735631</v>
       </c>
       <c r="C322" t="n">
-        <v>44757.0364176621</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="323">
@@ -7829,10 +7829,10 @@
         <v>5493</v>
       </c>
       <c r="B335" t="n">
-        <v>1890.661705562889</v>
+        <v>1890.661705562905</v>
       </c>
       <c r="C335" t="n">
-        <v>6796.505323276539</v>
+        <v>6796.505323276597</v>
       </c>
     </row>
     <row r="336">
@@ -7851,10 +7851,10 @@
         <v>5495</v>
       </c>
       <c r="B337" t="n">
-        <v>0</v>
+        <v>1856.899955603446</v>
       </c>
       <c r="C337" t="n">
-        <v>0</v>
+        <v>6675.139394804332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New plots added for each stage of the optimization
</commit_message>
<xml_diff>
--- a/first_stage_optimization/lshp_operation.xlsx
+++ b/first_stage_optimization/lshp_operation.xlsx
@@ -439,10 +439,10 @@
         <v>288</v>
       </c>
       <c r="B2" t="n">
-        <v>11197.08202174817</v>
+        <v>12937.01956816348</v>
       </c>
       <c r="C2" t="n">
-        <v>30882.6047416915</v>
+        <v>35681.5160488343</v>
       </c>
     </row>
     <row r="3">
@@ -450,10 +450,10 @@
         <v>289</v>
       </c>
       <c r="B3" t="n">
-        <v>16134.66738214708</v>
+        <v>16134.66738214692</v>
       </c>
       <c r="C3" t="n">
-        <v>44500.92929869557</v>
+        <v>44500.92929869513</v>
       </c>
     </row>
     <row r="4">
@@ -494,10 +494,10 @@
         <v>293</v>
       </c>
       <c r="B7" t="n">
-        <v>15640.50738895312</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C7" t="n">
-        <v>43137.98958642726</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="8">
@@ -505,10 +505,10 @@
         <v>294</v>
       </c>
       <c r="B8" t="n">
-        <v>15771.71513208502</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C8" t="n">
-        <v>43499.8728755129</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="9">
@@ -538,10 +538,10 @@
         <v>297</v>
       </c>
       <c r="B11" t="n">
-        <v>7427.29319618396</v>
+        <v>9167.230742599275</v>
       </c>
       <c r="C11" t="n">
-        <v>20485.1728006358</v>
+        <v>25284.0841077786</v>
       </c>
     </row>
     <row r="12">
@@ -549,10 +549,10 @@
         <v>298</v>
       </c>
       <c r="B12" t="n">
-        <v>2671.138940993995</v>
+        <v>4411.076487409309</v>
       </c>
       <c r="C12" t="n">
-        <v>7367.252286321891</v>
+        <v>12166.16359346469</v>
       </c>
     </row>
     <row r="13">
@@ -571,10 +571,10 @@
         <v>300</v>
       </c>
       <c r="B14" t="n">
-        <v>11725.51941396181</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C14" t="n">
-        <v>32340.08474253159</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="15">
@@ -582,10 +582,10 @@
         <v>301</v>
       </c>
       <c r="B15" t="n">
-        <v>16134.66738214708</v>
+        <v>16031.5577692864</v>
       </c>
       <c r="C15" t="n">
-        <v>44500.92929869557</v>
+        <v>44216.5432941222</v>
       </c>
     </row>
     <row r="16">
@@ -648,10 +648,10 @@
         <v>307</v>
       </c>
       <c r="B21" t="n">
-        <v>2420.200107322064</v>
+        <v>3903.493971266206</v>
       </c>
       <c r="C21" t="n">
-        <v>6675.139394804341</v>
+        <v>10766.20330118549</v>
       </c>
     </row>
     <row r="22">
@@ -659,10 +659,10 @@
         <v>308</v>
       </c>
       <c r="B22" t="n">
-        <v>3442.235445494172</v>
+        <v>5182.172991909332</v>
       </c>
       <c r="C22" t="n">
-        <v>9494.008928804804</v>
+        <v>14292.92023594718</v>
       </c>
     </row>
     <row r="23">
@@ -670,10 +670,10 @@
         <v>309</v>
       </c>
       <c r="B23" t="n">
-        <v>8223.007242495609</v>
+        <v>16134.66738214692</v>
       </c>
       <c r="C23" t="n">
-        <v>22679.82693748368</v>
+        <v>44500.92929869513</v>
       </c>
     </row>
     <row r="24">
@@ -681,10 +681,10 @@
         <v>310</v>
       </c>
       <c r="B24" t="n">
-        <v>12332.30114269007</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C24" t="n">
-        <v>34013.64578784662</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="25">
@@ -703,10 +703,10 @@
         <v>312</v>
       </c>
       <c r="B26" t="n">
-        <v>14184.39603300014</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C26" t="n">
-        <v>39121.8975922415</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="27">
@@ -736,10 +736,10 @@
         <v>315</v>
       </c>
       <c r="B29" t="n">
-        <v>15700.36452466098</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C29" t="n">
-        <v>43303.08119328029</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="30">
@@ -769,10 +769,10 @@
         <v>318</v>
       </c>
       <c r="B32" t="n">
-        <v>15771.71513208502</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C32" t="n">
-        <v>43499.8728755129</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="33">
@@ -780,10 +780,10 @@
         <v>319</v>
       </c>
       <c r="B33" t="n">
-        <v>4574.87140815473</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C33" t="n">
-        <v>12617.92538160311</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="34">
@@ -813,10 +813,10 @@
         <v>322</v>
       </c>
       <c r="B36" t="n">
-        <v>5106.013640195039</v>
+        <v>6845.951186610199</v>
       </c>
       <c r="C36" t="n">
-        <v>14082.8655849401</v>
+        <v>18881.77689208247</v>
       </c>
     </row>
     <row r="37">
@@ -824,10 +824,10 @@
         <v>323</v>
       </c>
       <c r="B37" t="n">
-        <v>2420.200107322064</v>
+        <v>13751.78979370113</v>
       </c>
       <c r="C37" t="n">
-        <v>6675.139394804341</v>
+        <v>37928.72891926834</v>
       </c>
     </row>
     <row r="38">
@@ -934,10 +934,10 @@
         <v>333</v>
       </c>
       <c r="B47" t="n">
-        <v>5546.398661717728</v>
+        <v>7286.336208132883</v>
       </c>
       <c r="C47" t="n">
-        <v>15297.4888704917</v>
+        <v>20096.40017763406</v>
       </c>
     </row>
     <row r="48">
@@ -945,10 +945,10 @@
         <v>334</v>
       </c>
       <c r="B48" t="n">
-        <v>12332.30114269007</v>
+        <v>14072.23868910538</v>
       </c>
       <c r="C48" t="n">
-        <v>34013.64578784662</v>
+        <v>38812.55709498942</v>
       </c>
     </row>
     <row r="49">
@@ -956,10 +956,10 @@
         <v>335</v>
       </c>
       <c r="B49" t="n">
-        <v>13180.5251643192</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C49" t="n">
-        <v>36353.12737255779</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="50">
@@ -967,10 +967,10 @@
         <v>336</v>
       </c>
       <c r="B50" t="n">
-        <v>11197.08202174817</v>
+        <v>16134.66738214188</v>
       </c>
       <c r="C50" t="n">
-        <v>30882.6047416915</v>
+        <v>44500.92929868122</v>
       </c>
     </row>
     <row r="51">
@@ -1011,10 +1011,10 @@
         <v>340</v>
       </c>
       <c r="B54" t="n">
-        <v>16134.66738214708</v>
+        <v>16134.66738214695</v>
       </c>
       <c r="C54" t="n">
-        <v>44500.92929869557</v>
+        <v>44500.92929869522</v>
       </c>
     </row>
     <row r="55">
@@ -1022,10 +1022,10 @@
         <v>341</v>
       </c>
       <c r="B55" t="n">
-        <v>13873.55516262652</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C55" t="n">
-        <v>38264.56925270922</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="56">
@@ -1033,10 +1033,10 @@
         <v>342</v>
       </c>
       <c r="B56" t="n">
-        <v>9891.411429789443</v>
+        <v>11631.34897620476</v>
       </c>
       <c r="C56" t="n">
-        <v>27281.44251603368</v>
+        <v>32080.35382317648</v>
       </c>
     </row>
     <row r="57">
@@ -1231,10 +1231,10 @@
         <v>360</v>
       </c>
       <c r="B74" t="n">
-        <v>0</v>
+        <v>2420.200107322061</v>
       </c>
       <c r="C74" t="n">
-        <v>0</v>
+        <v>6675.139394804333</v>
       </c>
     </row>
     <row r="75">
@@ -1242,10 +1242,10 @@
         <v>361</v>
       </c>
       <c r="B75" t="n">
-        <v>2420.200107322062</v>
+        <v>2420.200107322061</v>
       </c>
       <c r="C75" t="n">
-        <v>6675.139394804335</v>
+        <v>6675.139394804333</v>
       </c>
     </row>
     <row r="76">
@@ -1253,10 +1253,10 @@
         <v>362</v>
       </c>
       <c r="B76" t="n">
-        <v>2420.200107322062</v>
+        <v>2420.200107322061</v>
       </c>
       <c r="C76" t="n">
-        <v>6675.139394804335</v>
+        <v>6675.139394804333</v>
       </c>
     </row>
     <row r="77">
@@ -1264,10 +1264,10 @@
         <v>363</v>
       </c>
       <c r="B77" t="n">
-        <v>2420.200107322064</v>
+        <v>12239.10204538795</v>
       </c>
       <c r="C77" t="n">
-        <v>6675.139394804341</v>
+        <v>33756.59391677224</v>
       </c>
     </row>
     <row r="78">
@@ -1275,10 +1275,10 @@
         <v>364</v>
       </c>
       <c r="B78" t="n">
-        <v>0</v>
+        <v>2938.65569474311</v>
       </c>
       <c r="C78" t="n">
-        <v>0</v>
+        <v>8105.088639736801</v>
       </c>
     </row>
     <row r="79">
@@ -1286,10 +1286,10 @@
         <v>365</v>
       </c>
       <c r="B79" t="n">
-        <v>2420.200107322062</v>
+        <v>3270.073686704226</v>
       </c>
       <c r="C79" t="n">
-        <v>6675.139394804335</v>
+        <v>9019.170614856805</v>
       </c>
     </row>
     <row r="80">
@@ -1297,10 +1297,10 @@
         <v>366</v>
       </c>
       <c r="B80" t="n">
-        <v>2420.200107322062</v>
+        <v>3743.795156917129</v>
       </c>
       <c r="C80" t="n">
-        <v>6675.139394804335</v>
+        <v>10325.73895952219</v>
       </c>
     </row>
     <row r="81">
@@ -1495,10 +1495,10 @@
         <v>384</v>
       </c>
       <c r="B98" t="n">
-        <v>2719.037683477357</v>
+        <v>4458.975229892671</v>
       </c>
       <c r="C98" t="n">
-        <v>7499.361520572798</v>
+        <v>12298.2728277156</v>
       </c>
     </row>
     <row r="99">
@@ -1506,10 +1506,10 @@
         <v>385</v>
       </c>
       <c r="B99" t="n">
-        <v>2990.384331759942</v>
+        <v>4730.321878175111</v>
       </c>
       <c r="C99" t="n">
-        <v>8247.761083121106</v>
+        <v>13046.67239026351</v>
       </c>
     </row>
     <row r="100">
@@ -1517,10 +1517,10 @@
         <v>386</v>
       </c>
       <c r="B100" t="n">
-        <v>3268.251465062969</v>
+        <v>4924.58664359358</v>
       </c>
       <c r="C100" t="n">
-        <v>9014.144756281385</v>
+        <v>13582.47287417559</v>
       </c>
     </row>
     <row r="101">
@@ -1528,10 +1528,10 @@
         <v>387</v>
       </c>
       <c r="B101" t="n">
-        <v>6948.505853923947</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C101" t="n">
-        <v>19164.63230467252</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="102">
@@ -1539,10 +1539,10 @@
         <v>388</v>
       </c>
       <c r="B102" t="n">
-        <v>2420.200107322062</v>
+        <v>5048.578090239315</v>
       </c>
       <c r="C102" t="n">
-        <v>6675.139394804335</v>
+        <v>13924.45293922051</v>
       </c>
     </row>
     <row r="103">
@@ -1550,10 +1550,10 @@
         <v>389</v>
       </c>
       <c r="B103" t="n">
-        <v>2420.200107322062</v>
+        <v>3270.073686704226</v>
       </c>
       <c r="C103" t="n">
-        <v>6675.139394804335</v>
+        <v>9019.170614856805</v>
       </c>
     </row>
     <row r="104">
@@ -1561,10 +1561,10 @@
         <v>390</v>
       </c>
       <c r="B104" t="n">
-        <v>4488.21056262738</v>
+        <v>6228.148109042694</v>
       </c>
       <c r="C104" t="n">
-        <v>12378.9066235192</v>
+        <v>17177.817930662</v>
       </c>
     </row>
     <row r="105">
@@ -1726,10 +1726,10 @@
         <v>405</v>
       </c>
       <c r="B119" t="n">
-        <v>2420.200107322062</v>
+        <v>2420.200107322061</v>
       </c>
       <c r="C119" t="n">
-        <v>6675.139394804335</v>
+        <v>6675.139394804333</v>
       </c>
     </row>
     <row r="120">
@@ -1737,10 +1737,10 @@
         <v>406</v>
       </c>
       <c r="B120" t="n">
-        <v>4074.021233385152</v>
+        <v>5813.958779800466</v>
       </c>
       <c r="C120" t="n">
-        <v>11236.53351967219</v>
+        <v>16035.44482681499</v>
       </c>
     </row>
     <row r="121">
@@ -1748,10 +1748,10 @@
         <v>407</v>
       </c>
       <c r="B121" t="n">
-        <v>4687.376665780643</v>
+        <v>6427.314212195957</v>
       </c>
       <c r="C121" t="n">
-        <v>12928.2254576296</v>
+        <v>17727.1367647724</v>
       </c>
     </row>
     <row r="122">
@@ -1759,10 +1759,10 @@
         <v>408</v>
       </c>
       <c r="B122" t="n">
-        <v>6621.629542051171</v>
+        <v>8361.567088466487</v>
       </c>
       <c r="C122" t="n">
-        <v>18263.07671015408</v>
+        <v>23061.98801729688</v>
       </c>
     </row>
     <row r="123">
@@ -1770,10 +1770,10 @@
         <v>409</v>
       </c>
       <c r="B123" t="n">
-        <v>6819.851204685992</v>
+        <v>8559.788751101307</v>
       </c>
       <c r="C123" t="n">
-        <v>18809.79068853721</v>
+        <v>23608.70199568001</v>
       </c>
     </row>
     <row r="124">
@@ -1781,10 +1781,10 @@
         <v>410</v>
       </c>
       <c r="B124" t="n">
-        <v>7099.280057115846</v>
+        <v>8839.21760353116</v>
       </c>
       <c r="C124" t="n">
-        <v>19580.48172985087</v>
+        <v>24379.39303699367</v>
       </c>
     </row>
     <row r="125">
@@ -1792,10 +1792,10 @@
         <v>411</v>
       </c>
       <c r="B125" t="n">
-        <v>7496.823652848921</v>
+        <v>9236.761199264234</v>
       </c>
       <c r="C125" t="n">
-        <v>20676.94433598069</v>
+        <v>25475.85564312349</v>
       </c>
     </row>
     <row r="126">
@@ -1803,10 +1803,10 @@
         <v>412</v>
       </c>
       <c r="B126" t="n">
-        <v>5654.012943367195</v>
+        <v>11339.74663090383</v>
       </c>
       <c r="C126" t="n">
-        <v>15594.2991750234</v>
+        <v>31276.08714421606</v>
       </c>
     </row>
     <row r="127">
@@ -1814,10 +1814,10 @@
         <v>413</v>
       </c>
       <c r="B127" t="n">
-        <v>4015.178821929269</v>
+        <v>5755.116368344424</v>
       </c>
       <c r="C127" t="n">
-        <v>11074.24061769019</v>
+        <v>15873.15192483255</v>
       </c>
     </row>
     <row r="128">
@@ -1825,10 +1825,10 @@
         <v>414</v>
       </c>
       <c r="B128" t="n">
-        <v>3070.942907548726</v>
+        <v>4810.88045396404</v>
       </c>
       <c r="C128" t="n">
-        <v>8469.949207652695</v>
+        <v>13268.86051479549</v>
       </c>
     </row>
     <row r="129">
@@ -1836,10 +1836,10 @@
         <v>415</v>
       </c>
       <c r="B129" t="n">
-        <v>2686.116864027475</v>
+        <v>4426.054410442789</v>
       </c>
       <c r="C129" t="n">
-        <v>7408.562805972993</v>
+        <v>12207.47411311579</v>
       </c>
     </row>
     <row r="130">
@@ -1847,10 +1847,10 @@
         <v>416</v>
       </c>
       <c r="B130" t="n">
-        <v>2574.019573866587</v>
+        <v>4313.957120281902</v>
       </c>
       <c r="C130" t="n">
-        <v>7099.38794256399</v>
+        <v>11898.29924970679</v>
       </c>
     </row>
     <row r="131">
@@ -1858,10 +1858,10 @@
         <v>417</v>
       </c>
       <c r="B131" t="n">
-        <v>2420.200107322064</v>
+        <v>4131.024741728158</v>
       </c>
       <c r="C131" t="n">
-        <v>6675.139394804341</v>
+        <v>11393.75455401198</v>
       </c>
     </row>
     <row r="132">
@@ -1869,10 +1869,10 @@
         <v>418</v>
       </c>
       <c r="B132" t="n">
-        <v>0</v>
+        <v>2475.240439975179</v>
       </c>
       <c r="C132" t="n">
-        <v>0</v>
+        <v>6826.9458060529</v>
       </c>
     </row>
     <row r="133">
@@ -1979,10 +1979,10 @@
         <v>428</v>
       </c>
       <c r="B142" t="n">
-        <v>2420.200107322062</v>
+        <v>3540.636238494415</v>
       </c>
       <c r="C142" t="n">
-        <v>6675.139394804335</v>
+        <v>9765.407565574016</v>
       </c>
     </row>
     <row r="143">
@@ -1990,10 +1990,10 @@
         <v>429</v>
       </c>
       <c r="B143" t="n">
-        <v>2607.407254098156</v>
+        <v>4347.344800513471</v>
       </c>
       <c r="C143" t="n">
-        <v>7191.4743030846</v>
+        <v>11990.3856102274</v>
       </c>
     </row>
     <row r="144">
@@ -2001,10 +2001,10 @@
         <v>430</v>
       </c>
       <c r="B144" t="n">
-        <v>3927.656650606756</v>
+        <v>5667.59419702207</v>
       </c>
       <c r="C144" t="n">
-        <v>10832.84624209859</v>
+        <v>15631.75754924139</v>
       </c>
     </row>
     <row r="145">
@@ -2012,10 +2012,10 @@
         <v>431</v>
       </c>
       <c r="B145" t="n">
-        <v>5076.471721924955</v>
+        <v>6816.40926834027</v>
       </c>
       <c r="C145" t="n">
-        <v>14001.38619741089</v>
+        <v>18800.29750455369</v>
       </c>
     </row>
     <row r="146">
@@ -2023,10 +2023,10 @@
         <v>432</v>
       </c>
       <c r="B146" t="n">
-        <v>6827.201907076305</v>
+        <v>8567.13945349162</v>
       </c>
       <c r="C146" t="n">
-        <v>18830.06461669572</v>
+        <v>23628.97592383852</v>
       </c>
     </row>
     <row r="147">
@@ -2034,10 +2034,10 @@
         <v>433</v>
       </c>
       <c r="B147" t="n">
-        <v>7561.883712310421</v>
+        <v>9301.821258725737</v>
       </c>
       <c r="C147" t="n">
-        <v>20856.3860956211</v>
+        <v>25655.2974027639</v>
       </c>
     </row>
     <row r="148">
@@ -2045,10 +2045,10 @@
         <v>434</v>
       </c>
       <c r="B148" t="n">
-        <v>7829.974092509725</v>
+        <v>9569.911638925039</v>
       </c>
       <c r="C148" t="n">
-        <v>21595.80456470652</v>
+        <v>26394.71587184932</v>
       </c>
     </row>
     <row r="149">
@@ -2056,10 +2056,10 @@
         <v>435</v>
       </c>
       <c r="B149" t="n">
-        <v>7982.762821060161</v>
+        <v>9722.700367475476</v>
       </c>
       <c r="C149" t="n">
-        <v>22017.2102401891</v>
+        <v>26816.1215473319</v>
       </c>
     </row>
     <row r="150">
@@ -2067,10 +2067,10 @@
         <v>436</v>
       </c>
       <c r="B150" t="n">
-        <v>7680.581968994567</v>
+        <v>9420.519515409724</v>
       </c>
       <c r="C150" t="n">
-        <v>21183.7670451921</v>
+        <v>25982.67835233447</v>
       </c>
     </row>
     <row r="151">
@@ -2078,10 +2078,10 @@
         <v>437</v>
       </c>
       <c r="B151" t="n">
-        <v>9781.100191118503</v>
+        <v>11521.03773753382</v>
       </c>
       <c r="C151" t="n">
-        <v>26977.1937505228</v>
+        <v>31776.1050576656</v>
       </c>
     </row>
     <row r="152">
@@ -2089,10 +2089,10 @@
         <v>438</v>
       </c>
       <c r="B152" t="n">
-        <v>5809.303108874029</v>
+        <v>7549.240655289194</v>
       </c>
       <c r="C152" t="n">
-        <v>16022.60404876681</v>
+        <v>20821.5153559092</v>
       </c>
     </row>
     <row r="153">
@@ -2100,10 +2100,10 @@
         <v>439</v>
       </c>
       <c r="B153" t="n">
-        <v>5438.630385589105</v>
+        <v>7178.567932004261</v>
       </c>
       <c r="C153" t="n">
-        <v>15000.25383471099</v>
+        <v>19799.16514185336</v>
       </c>
     </row>
     <row r="154">
@@ -2111,10 +2111,10 @@
         <v>440</v>
       </c>
       <c r="B154" t="n">
-        <v>5318.157006129553</v>
+        <v>6974.492184660128</v>
       </c>
       <c r="C154" t="n">
-        <v>14667.97692966388</v>
+        <v>19236.30504755799</v>
       </c>
     </row>
     <row r="155">
@@ -2122,10 +2122,10 @@
         <v>441</v>
       </c>
       <c r="B155" t="n">
-        <v>3430.999798591454</v>
+        <v>5087.334977122176</v>
       </c>
       <c r="C155" t="n">
-        <v>9463.019958496297</v>
+        <v>14031.34807639081</v>
       </c>
     </row>
     <row r="156">
@@ -2133,10 +2133,10 @@
         <v>442</v>
       </c>
       <c r="B156" t="n">
-        <v>2420.200107322064</v>
+        <v>4011.467085957548</v>
       </c>
       <c r="C156" t="n">
-        <v>6675.139394804341</v>
+        <v>11064.003300977</v>
       </c>
     </row>
     <row r="157">
@@ -2155,10 +2155,10 @@
         <v>444</v>
       </c>
       <c r="B158" t="n">
-        <v>7731.830712880651</v>
+        <v>16134.66738214707</v>
       </c>
       <c r="C158" t="n">
-        <v>21325.11589821185</v>
+        <v>44500.92929869554</v>
       </c>
     </row>
     <row r="159">
@@ -2265,10 +2265,10 @@
         <v>454</v>
       </c>
       <c r="B168" t="n">
-        <v>2420.200107322064</v>
+        <v>3821.739505649951</v>
       </c>
       <c r="C168" t="n">
-        <v>6675.139394804341</v>
+        <v>10540.7168000961</v>
       </c>
     </row>
     <row r="169">
@@ -2276,10 +2276,10 @@
         <v>455</v>
       </c>
       <c r="B169" t="n">
-        <v>2788.370147238635</v>
+        <v>4528.307693653949</v>
       </c>
       <c r="C169" t="n">
-        <v>7690.586972877994</v>
+        <v>12489.49828002079</v>
       </c>
     </row>
     <row r="170">
@@ -2287,10 +2287,10 @@
         <v>456</v>
       </c>
       <c r="B170" t="n">
-        <v>2719.037683477357</v>
+        <v>4458.975229892671</v>
       </c>
       <c r="C170" t="n">
-        <v>7499.361520572798</v>
+        <v>12298.2728277156</v>
       </c>
     </row>
     <row r="171">
@@ -2298,10 +2298,10 @@
         <v>457</v>
       </c>
       <c r="B171" t="n">
-        <v>2990.384331759942</v>
+        <v>4730.321878175097</v>
       </c>
       <c r="C171" t="n">
-        <v>8247.761083121106</v>
+        <v>13046.67239026347</v>
       </c>
     </row>
     <row r="172">
@@ -2309,10 +2309,10 @@
         <v>458</v>
       </c>
       <c r="B172" t="n">
-        <v>3268.251465062969</v>
+        <v>5008.189011478284</v>
       </c>
       <c r="C172" t="n">
-        <v>9014.144756281385</v>
+        <v>13813.05606342418</v>
       </c>
     </row>
     <row r="173">
@@ -2320,10 +2320,10 @@
         <v>459</v>
       </c>
       <c r="B173" t="n">
-        <v>3800.567685719266</v>
+        <v>5540.50523213458</v>
       </c>
       <c r="C173" t="n">
-        <v>10482.32293057619</v>
+        <v>15281.23423771899</v>
       </c>
     </row>
     <row r="174">
@@ -2331,10 +2331,10 @@
         <v>460</v>
       </c>
       <c r="B174" t="n">
-        <v>9477.803061384062</v>
+        <v>11217.74060779926</v>
       </c>
       <c r="C174" t="n">
-        <v>26140.67175678501</v>
+        <v>30939.58306392749</v>
       </c>
     </row>
     <row r="175">
@@ -2342,10 +2342,10 @@
         <v>461</v>
       </c>
       <c r="B175" t="n">
-        <v>9610.512602761624</v>
+        <v>11350.45014917682</v>
       </c>
       <c r="C175" t="n">
-        <v>26506.69714660122</v>
+        <v>31305.60845374369</v>
       </c>
     </row>
     <row r="176">
@@ -2353,10 +2353,10 @@
         <v>462</v>
       </c>
       <c r="B176" t="n">
-        <v>9891.411429789443</v>
+        <v>11631.34897620476</v>
       </c>
       <c r="C176" t="n">
-        <v>27281.44251603368</v>
+        <v>32080.35382317648</v>
       </c>
     </row>
     <row r="177">
@@ -2529,10 +2529,10 @@
         <v>478</v>
       </c>
       <c r="B192" t="n">
-        <v>0</v>
+        <v>3347.955278995932</v>
       </c>
       <c r="C192" t="n">
-        <v>0</v>
+        <v>9233.975367267005</v>
       </c>
     </row>
     <row r="193">
@@ -2540,10 +2540,10 @@
         <v>479</v>
       </c>
       <c r="B193" t="n">
-        <v>2420.200107322064</v>
+        <v>3834.478953229075</v>
       </c>
       <c r="C193" t="n">
-        <v>6675.139394804341</v>
+        <v>10575.85339402739</v>
       </c>
     </row>
     <row r="194">
@@ -2551,10 +2551,10 @@
         <v>480</v>
       </c>
       <c r="B194" t="n">
-        <v>2719.037683477357</v>
+        <v>4458.975229892671</v>
       </c>
       <c r="C194" t="n">
-        <v>7499.361520572798</v>
+        <v>12298.2728277156</v>
       </c>
     </row>
     <row r="195">
@@ -2562,10 +2562,10 @@
         <v>481</v>
       </c>
       <c r="B195" t="n">
-        <v>2990.384331759942</v>
+        <v>4646.71951029074</v>
       </c>
       <c r="C195" t="n">
-        <v>8247.761083121106</v>
+        <v>12816.08920101583</v>
       </c>
     </row>
     <row r="196">
@@ -2573,10 +2573,10 @@
         <v>482</v>
       </c>
       <c r="B196" t="n">
-        <v>3268.251465062969</v>
+        <v>9167.273969977028</v>
       </c>
       <c r="C196" t="n">
-        <v>9014.144756281385</v>
+        <v>25284.20333294982</v>
       </c>
     </row>
     <row r="197">
@@ -2584,10 +2584,10 @@
         <v>483</v>
       </c>
       <c r="B197" t="n">
-        <v>3800.567685719266</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C197" t="n">
-        <v>10482.32293057619</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="198">
@@ -2595,10 +2595,10 @@
         <v>484</v>
       </c>
       <c r="B198" t="n">
-        <v>6512.570198329713</v>
+        <v>16134.66738214708</v>
       </c>
       <c r="C198" t="n">
-        <v>17962.28078859199</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="199">
@@ -2606,10 +2606,10 @@
         <v>485</v>
       </c>
       <c r="B199" t="n">
-        <v>6706.333521350718</v>
+        <v>8446.271067766033</v>
       </c>
       <c r="C199" t="n">
-        <v>18496.69824723629</v>
+        <v>23295.60955437909</v>
       </c>
     </row>
     <row r="200">
@@ -2617,10 +2617,10 @@
         <v>486</v>
       </c>
       <c r="B200" t="n">
-        <v>7042.425069744652</v>
+        <v>8782.362616159966</v>
       </c>
       <c r="C200" t="n">
-        <v>19423.67033031231</v>
+        <v>24222.58163745511</v>
       </c>
     </row>
     <row r="201">
@@ -2782,10 +2782,10 @@
         <v>501</v>
       </c>
       <c r="B215" t="n">
-        <v>2420.200107322062</v>
+        <v>2420.200107322061</v>
       </c>
       <c r="C215" t="n">
-        <v>6675.139394804335</v>
+        <v>6675.139394804333</v>
       </c>
     </row>
     <row r="216">
@@ -2793,10 +2793,10 @@
         <v>502</v>
       </c>
       <c r="B216" t="n">
-        <v>0</v>
+        <v>3347.955278995932</v>
       </c>
       <c r="C216" t="n">
-        <v>0</v>
+        <v>9233.975367267005</v>
       </c>
     </row>
     <row r="217">
@@ -2804,10 +2804,10 @@
         <v>503</v>
       </c>
       <c r="B217" t="n">
-        <v>2420.200107322064</v>
+        <v>3834.478953229075</v>
       </c>
       <c r="C217" t="n">
-        <v>6675.139394804341</v>
+        <v>10575.85339402739</v>
       </c>
     </row>
     <row r="218">
@@ -2815,10 +2815,10 @@
         <v>504</v>
       </c>
       <c r="B218" t="n">
-        <v>2719.037683477357</v>
+        <v>4458.97522989251</v>
       </c>
       <c r="C218" t="n">
-        <v>7499.361520572798</v>
+        <v>12298.27282771515</v>
       </c>
     </row>
     <row r="219">
@@ -2826,10 +2826,10 @@
         <v>505</v>
       </c>
       <c r="B219" t="n">
-        <v>2990.384331759942</v>
+        <v>4730.321878175257</v>
       </c>
       <c r="C219" t="n">
-        <v>8247.761083121106</v>
+        <v>13046.67239026391</v>
       </c>
     </row>
     <row r="220">
@@ -2837,10 +2837,10 @@
         <v>506</v>
       </c>
       <c r="B220" t="n">
-        <v>5970.788395873496</v>
+        <v>7710.725942288811</v>
       </c>
       <c r="C220" t="n">
-        <v>16467.99564992831</v>
+        <v>21266.90695707111</v>
       </c>
     </row>
     <row r="221">
@@ -2848,10 +2848,10 @@
         <v>507</v>
       </c>
       <c r="B221" t="n">
-        <v>6480.875291557313</v>
+        <v>8220.812837972628</v>
       </c>
       <c r="C221" t="n">
-        <v>17874.86325639248</v>
+        <v>22673.77456353528</v>
       </c>
     </row>
     <row r="222">
@@ -2859,10 +2859,10 @@
         <v>508</v>
       </c>
       <c r="B222" t="n">
-        <v>6512.570198329713</v>
+        <v>8252.507744745028</v>
       </c>
       <c r="C222" t="n">
-        <v>17962.28078859199</v>
+        <v>22761.19209573479</v>
       </c>
     </row>
     <row r="223">
@@ -2870,10 +2870,10 @@
         <v>509</v>
       </c>
       <c r="B223" t="n">
-        <v>6706.333521350718</v>
+        <v>8446.271067766033</v>
       </c>
       <c r="C223" t="n">
-        <v>18496.69824723629</v>
+        <v>23295.60955437909</v>
       </c>
     </row>
     <row r="224">
@@ -2881,10 +2881,10 @@
         <v>510</v>
       </c>
       <c r="B224" t="n">
-        <v>4488.21056262738</v>
+        <v>6228.148109042542</v>
       </c>
       <c r="C224" t="n">
-        <v>12378.9066235192</v>
+        <v>17177.81793066158</v>
       </c>
     </row>
     <row r="225">
@@ -4014,10 +4014,10 @@
         <v>613</v>
       </c>
       <c r="B327" t="n">
-        <v>2420.200107322064</v>
+        <v>0</v>
       </c>
       <c r="C327" t="n">
-        <v>6675.139394804341</v>
+        <v>0</v>
       </c>
     </row>
     <row r="328">
@@ -4298,10 +4298,10 @@
         <v>5172</v>
       </c>
       <c r="B14" t="n">
-        <v>7563.007057174681</v>
+        <v>12379.33303735647</v>
       </c>
       <c r="C14" t="n">
-        <v>27187.31625696217</v>
+        <v>44500.92929869613</v>
       </c>
     </row>
     <row r="15">
@@ -4408,10 +4408,10 @@
         <v>5182</v>
       </c>
       <c r="B24" t="n">
-        <v>1874.820568382665</v>
+        <v>8915.784984633759</v>
       </c>
       <c r="C24" t="n">
-        <v>6739.55998352836</v>
+        <v>32050.2498839218</v>
       </c>
     </row>
     <row r="25">
@@ -4419,10 +4419,10 @@
         <v>5183</v>
       </c>
       <c r="B25" t="n">
-        <v>1856.899955603442</v>
+        <v>1856.899955603446</v>
       </c>
       <c r="C25" t="n">
-        <v>6675.139394804318</v>
+        <v>6675.139394804333</v>
       </c>
     </row>
     <row r="26">
@@ -4441,10 +4441,10 @@
         <v>5185</v>
       </c>
       <c r="B27" t="n">
-        <v>2284.204171165625</v>
+        <v>2284.204171165599</v>
       </c>
       <c r="C27" t="n">
-        <v>8211.202333606079</v>
+        <v>8211.202333605986</v>
       </c>
     </row>
     <row r="28">
@@ -4463,10 +4463,10 @@
         <v>5187</v>
       </c>
       <c r="B29" t="n">
-        <v>2299.850630719266</v>
+        <v>2299.85063071924</v>
       </c>
       <c r="C29" t="n">
-        <v>8267.447850894478</v>
+        <v>8267.447850894387</v>
       </c>
     </row>
     <row r="30">
@@ -4474,10 +4474,10 @@
         <v>5188</v>
       </c>
       <c r="B30" t="n">
-        <v>9272.421191446763</v>
+        <v>12379.33303735646</v>
       </c>
       <c r="C30" t="n">
-        <v>33332.27716090422</v>
+        <v>44500.92929869612</v>
       </c>
     </row>
     <row r="31">
@@ -4485,10 +4485,10 @@
         <v>5189</v>
       </c>
       <c r="B31" t="n">
-        <v>1856.899955603447</v>
+        <v>0</v>
       </c>
       <c r="C31" t="n">
-        <v>6675.139394804335</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -4496,10 +4496,10 @@
         <v>5190</v>
       </c>
       <c r="B32" t="n">
-        <v>2070.628765404943</v>
+        <v>2070.62876540492</v>
       </c>
       <c r="C32" t="n">
-        <v>7443.44659078732</v>
+        <v>7443.446590787236</v>
       </c>
     </row>
     <row r="33">
@@ -4650,10 +4650,10 @@
         <v>5204</v>
       </c>
       <c r="B46" t="n">
-        <v>2346.064435599156</v>
+        <v>2346.06443559913</v>
       </c>
       <c r="C46" t="n">
-        <v>8433.57612754539</v>
+        <v>8433.576127545297</v>
       </c>
     </row>
     <row r="47">
@@ -4661,10 +4661,10 @@
         <v>5205</v>
       </c>
       <c r="B47" t="n">
-        <v>2157.297466391335</v>
+        <v>12379.33303735643</v>
       </c>
       <c r="C47" t="n">
-        <v>7755.001157044377</v>
+        <v>44500.92929869599</v>
       </c>
     </row>
     <row r="48">
@@ -4672,10 +4672,10 @@
         <v>5206</v>
       </c>
       <c r="B48" t="n">
-        <v>1874.820568382665</v>
+        <v>1874.82056838264</v>
       </c>
       <c r="C48" t="n">
-        <v>6739.55998352836</v>
+        <v>6739.55998352827</v>
       </c>
     </row>
     <row r="49">
@@ -4694,10 +4694,10 @@
         <v>5208</v>
       </c>
       <c r="B50" t="n">
-        <v>2552.756939774566</v>
+        <v>0</v>
       </c>
       <c r="C50" t="n">
-        <v>9176.589380935055</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -4705,10 +4705,10 @@
         <v>5209</v>
       </c>
       <c r="B51" t="n">
-        <v>2518.087048222285</v>
+        <v>2284.204171165599</v>
       </c>
       <c r="C51" t="n">
-        <v>9051.958886860313</v>
+        <v>8211.202333605986</v>
       </c>
     </row>
     <row r="52">
@@ -4738,10 +4738,10 @@
         <v>5212</v>
       </c>
       <c r="B54" t="n">
-        <v>12379.33303735631</v>
+        <v>4470.603618251954</v>
       </c>
       <c r="C54" t="n">
-        <v>44500.92929869557</v>
+        <v>16070.81859240528</v>
       </c>
     </row>
     <row r="55">
@@ -4749,10 +4749,10 @@
         <v>5213</v>
       </c>
       <c r="B55" t="n">
-        <v>1856.899955603447</v>
+        <v>0</v>
       </c>
       <c r="C55" t="n">
-        <v>6675.139394804335</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -4793,10 +4793,10 @@
         <v>5217</v>
       </c>
       <c r="B59" t="n">
-        <v>1856.899955603447</v>
+        <v>0</v>
       </c>
       <c r="C59" t="n">
-        <v>6675.139394804335</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -4804,10 +4804,10 @@
         <v>5218</v>
       </c>
       <c r="B60" t="n">
-        <v>2205.349870521857</v>
+        <v>2205.349870521832</v>
       </c>
       <c r="C60" t="n">
-        <v>7927.738786155077</v>
+        <v>7927.738786154987</v>
       </c>
     </row>
     <row r="61">
@@ -4815,10 +4815,10 @@
         <v>5219</v>
       </c>
       <c r="B61" t="n">
-        <v>2033.817988805349</v>
+        <v>2132.385027743748</v>
       </c>
       <c r="C61" t="n">
-        <v>7311.120094525737</v>
+        <v>7665.446520492558</v>
       </c>
     </row>
     <row r="62">
@@ -4903,10 +4903,10 @@
         <v>5227</v>
       </c>
       <c r="B69" t="n">
-        <v>2268.320949722101</v>
+        <v>1856.899955603447</v>
       </c>
       <c r="C69" t="n">
-        <v>8154.105710358214</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="70">
@@ -4914,10 +4914,10 @@
         <v>5228</v>
       </c>
       <c r="B70" t="n">
-        <v>2346.064435599156</v>
+        <v>0</v>
       </c>
       <c r="C70" t="n">
-        <v>8433.57612754539</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -4925,10 +4925,10 @@
         <v>5229</v>
       </c>
       <c r="B71" t="n">
-        <v>2157.297466391335</v>
+        <v>0</v>
       </c>
       <c r="C71" t="n">
-        <v>7755.001157044377</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -5002,10 +5002,10 @@
         <v>5236</v>
       </c>
       <c r="B78" t="n">
-        <v>8662.985600275406</v>
+        <v>0</v>
       </c>
       <c r="C78" t="n">
-        <v>31141.49272421562</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -5200,10 +5200,10 @@
         <v>5254</v>
       </c>
       <c r="B96" t="n">
-        <v>1874.820568382665</v>
+        <v>1856.899955603447</v>
       </c>
       <c r="C96" t="n">
-        <v>6739.55998352836</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="97">
@@ -5222,10 +5222,10 @@
         <v>5256</v>
       </c>
       <c r="B98" t="n">
-        <v>0</v>
+        <v>1856.899955603447</v>
       </c>
       <c r="C98" t="n">
-        <v>0</v>
+        <v>6675.139394804337</v>
       </c>
     </row>
     <row r="99">
@@ -5233,10 +5233,10 @@
         <v>5257</v>
       </c>
       <c r="B99" t="n">
-        <v>0</v>
+        <v>1856.899955603445</v>
       </c>
       <c r="C99" t="n">
-        <v>0</v>
+        <v>6675.139394804329</v>
       </c>
     </row>
     <row r="100">
@@ -5244,10 +5244,10 @@
         <v>5258</v>
       </c>
       <c r="B100" t="n">
-        <v>0</v>
+        <v>9120.569383798414</v>
       </c>
       <c r="C100" t="n">
-        <v>0</v>
+        <v>32786.40392721332</v>
       </c>
     </row>
     <row r="101">
@@ -5255,10 +5255,10 @@
         <v>5259</v>
       </c>
       <c r="B101" t="n">
-        <v>0</v>
+        <v>1856.899955603445</v>
       </c>
       <c r="C101" t="n">
-        <v>0</v>
+        <v>6675.13939480433</v>
       </c>
     </row>
     <row r="102">
@@ -5266,10 +5266,10 @@
         <v>5260</v>
       </c>
       <c r="B102" t="n">
-        <v>12379.33303735631</v>
+        <v>0</v>
       </c>
       <c r="C102" t="n">
-        <v>44500.92929869557</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -5277,10 +5277,10 @@
         <v>5261</v>
       </c>
       <c r="B103" t="n">
-        <v>12379.33303735631</v>
+        <v>3147.954604277232</v>
       </c>
       <c r="C103" t="n">
-        <v>44500.92929869557</v>
+        <v>11316.19166054529</v>
       </c>
     </row>
     <row r="104">
@@ -5288,10 +5288,10 @@
         <v>5262</v>
       </c>
       <c r="B104" t="n">
-        <v>2070.628765404943</v>
+        <v>1856.899955603447</v>
       </c>
       <c r="C104" t="n">
-        <v>7443.44659078732</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="105">
@@ -5519,10 +5519,10 @@
         <v>5283</v>
       </c>
       <c r="B125" t="n">
-        <v>0</v>
+        <v>1856.899955603445</v>
       </c>
       <c r="C125" t="n">
-        <v>0</v>
+        <v>6675.13939480433</v>
       </c>
     </row>
     <row r="126">
@@ -5530,10 +5530,10 @@
         <v>5284</v>
       </c>
       <c r="B126" t="n">
-        <v>0</v>
+        <v>6709.015463848392</v>
       </c>
       <c r="C126" t="n">
-        <v>0</v>
+        <v>24117.40777307106</v>
       </c>
     </row>
     <row r="127">
@@ -5541,10 +5541,10 @@
         <v>5285</v>
       </c>
       <c r="B127" t="n">
-        <v>0</v>
+        <v>1856.899955603447</v>
       </c>
       <c r="C127" t="n">
-        <v>0</v>
+        <v>6675.139394804337</v>
       </c>
     </row>
     <row r="128">
@@ -5552,10 +5552,10 @@
         <v>5286</v>
       </c>
       <c r="B128" t="n">
-        <v>0</v>
+        <v>7516.445331520613</v>
       </c>
       <c r="C128" t="n">
-        <v>0</v>
+        <v>27019.93728306234</v>
       </c>
     </row>
     <row r="129">
@@ -5783,10 +5783,10 @@
         <v>5307</v>
       </c>
       <c r="B149" t="n">
-        <v>9800.278967776228</v>
+        <v>12379.33303735647</v>
       </c>
       <c r="C149" t="n">
-        <v>35229.80762666676</v>
+        <v>44500.92929869614</v>
       </c>
     </row>
     <row r="150">
@@ -5805,10 +5805,10 @@
         <v>5309</v>
       </c>
       <c r="B151" t="n">
-        <v>12379.33303735631</v>
+        <v>12379.33303735647</v>
       </c>
       <c r="C151" t="n">
-        <v>44500.92929869557</v>
+        <v>44500.92929869614</v>
       </c>
     </row>
     <row r="152">
@@ -6014,10 +6014,10 @@
         <v>5328</v>
       </c>
       <c r="B170" t="n">
-        <v>0</v>
+        <v>12379.33303735629</v>
       </c>
       <c r="C170" t="n">
-        <v>0</v>
+        <v>44500.9292986955</v>
       </c>
     </row>
     <row r="171">
@@ -6025,10 +6025,10 @@
         <v>5329</v>
       </c>
       <c r="B171" t="n">
-        <v>0</v>
+        <v>1856.899955603445</v>
       </c>
       <c r="C171" t="n">
-        <v>0</v>
+        <v>6675.139394804329</v>
       </c>
     </row>
     <row r="172">
@@ -6036,10 +6036,10 @@
         <v>5330</v>
       </c>
       <c r="B172" t="n">
-        <v>12379.33303735631</v>
+        <v>12379.33303735629</v>
       </c>
       <c r="C172" t="n">
-        <v>44500.92929869557</v>
+        <v>44500.92929869548</v>
       </c>
     </row>
     <row r="173">
@@ -6050,7 +6050,7 @@
         <v>12379.33303735631</v>
       </c>
       <c r="C173" t="n">
-        <v>44500.92929869556</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="174">
@@ -6058,10 +6058,10 @@
         <v>5332</v>
       </c>
       <c r="B174" t="n">
-        <v>5422.989787194354</v>
+        <v>12379.33303735619</v>
       </c>
       <c r="C174" t="n">
-        <v>19494.43353525137</v>
+        <v>44500.92929869511</v>
       </c>
     </row>
     <row r="175">
@@ -6069,10 +6069,10 @@
         <v>5333</v>
       </c>
       <c r="B175" t="n">
-        <v>0</v>
+        <v>1856.899955603446</v>
       </c>
       <c r="C175" t="n">
-        <v>0</v>
+        <v>6675.139394804333</v>
       </c>
     </row>
     <row r="176">
@@ -6080,10 +6080,10 @@
         <v>5334</v>
       </c>
       <c r="B176" t="n">
-        <v>2070.628765404943</v>
+        <v>2070.628765404715</v>
       </c>
       <c r="C176" t="n">
-        <v>7443.44659078732</v>
+        <v>7443.446590786497</v>
       </c>
     </row>
     <row r="177">
@@ -6091,10 +6091,10 @@
         <v>5335</v>
       </c>
       <c r="B177" t="n">
-        <v>1856.899955603447</v>
+        <v>0</v>
       </c>
       <c r="C177" t="n">
-        <v>6675.139394804335</v>
+        <v>0</v>
       </c>
     </row>
     <row r="178">
@@ -6300,10 +6300,10 @@
         <v>5354</v>
       </c>
       <c r="B196" t="n">
-        <v>12379.33303735631</v>
+        <v>12379.33303735647</v>
       </c>
       <c r="C196" t="n">
-        <v>44500.92929869557</v>
+        <v>44500.92929869613</v>
       </c>
     </row>
     <row r="197">
@@ -6322,10 +6322,10 @@
         <v>5356</v>
       </c>
       <c r="B198" t="n">
-        <v>0</v>
+        <v>1856.899955603444</v>
       </c>
       <c r="C198" t="n">
-        <v>0</v>
+        <v>6675.139394804326</v>
       </c>
     </row>
     <row r="199">
@@ -6333,10 +6333,10 @@
         <v>5357</v>
       </c>
       <c r="B199" t="n">
-        <v>0</v>
+        <v>12379.33303735647</v>
       </c>
       <c r="C199" t="n">
-        <v>0</v>
+        <v>44500.92929869614</v>
       </c>
     </row>
     <row r="200">
@@ -6344,10 +6344,10 @@
         <v>5358</v>
       </c>
       <c r="B200" t="n">
-        <v>2070.628765404943</v>
+        <v>4659.605940207125</v>
       </c>
       <c r="C200" t="n">
-        <v>7443.44659078732</v>
+        <v>16750.23960331401</v>
       </c>
     </row>
     <row r="201">
@@ -7367,10 +7367,10 @@
         <v>5451</v>
       </c>
       <c r="B293" t="n">
-        <v>12379.33303735631</v>
+        <v>8794.585734492903</v>
       </c>
       <c r="C293" t="n">
-        <v>44500.92929869557</v>
+        <v>31614.56572829746</v>
       </c>
     </row>
     <row r="294">
@@ -7378,10 +7378,10 @@
         <v>5452</v>
       </c>
       <c r="B294" t="n">
-        <v>2364.6056215037</v>
+        <v>1856.899955603448</v>
       </c>
       <c r="C294" t="n">
-        <v>8500.227537646582</v>
+        <v>6675.139394804339</v>
       </c>
     </row>
     <row r="295">
@@ -7389,10 +7389,10 @@
         <v>5453</v>
       </c>
       <c r="B295" t="n">
-        <v>1856.899955603448</v>
+        <v>1856.899955603447</v>
       </c>
       <c r="C295" t="n">
-        <v>6675.139394804341</v>
+        <v>6675.139394804337</v>
       </c>
     </row>
     <row r="296">
@@ -7565,10 +7565,10 @@
         <v>5469</v>
       </c>
       <c r="B311" t="n">
-        <v>2327.1776631764</v>
+        <v>2327.177663176375</v>
       </c>
       <c r="C311" t="n">
-        <v>8365.682411322605</v>
+        <v>8365.682411322516</v>
       </c>
     </row>
     <row r="312">
@@ -7598,10 +7598,10 @@
         <v>5472</v>
       </c>
       <c r="B314" t="n">
-        <v>1856.899955603442</v>
+        <v>1856.899955603446</v>
       </c>
       <c r="C314" t="n">
-        <v>6675.139394804317</v>
+        <v>6675.139394804331</v>
       </c>
     </row>
     <row r="315">
@@ -7620,10 +7620,10 @@
         <v>5474</v>
       </c>
       <c r="B316" t="n">
-        <v>1856.899955603447</v>
+        <v>1856.899955603445</v>
       </c>
       <c r="C316" t="n">
-        <v>6675.139394804335</v>
+        <v>6675.139394804328</v>
       </c>
     </row>
     <row r="317">
@@ -7631,10 +7631,10 @@
         <v>5475</v>
       </c>
       <c r="B317" t="n">
-        <v>7707.830164704253</v>
+        <v>12379.33303735631</v>
       </c>
       <c r="C317" t="n">
-        <v>27707.92288815489</v>
+        <v>44500.92929869557</v>
       </c>
     </row>
     <row r="318">
@@ -7642,10 +7642,10 @@
         <v>5476</v>
       </c>
       <c r="B318" t="n">
-        <v>1856.89995560341</v>
+        <v>8969.238617531319</v>
       </c>
       <c r="C318" t="n">
-        <v>6675.139394804203</v>
+        <v>32242.40372057476</v>
       </c>
     </row>
     <row r="319">
@@ -7653,10 +7653,10 @@
         <v>5477</v>
       </c>
       <c r="B319" t="n">
-        <v>0</v>
+        <v>1856.899955603446</v>
       </c>
       <c r="C319" t="n">
-        <v>0</v>
+        <v>6675.139394804331</v>
       </c>
     </row>
     <row r="320">
@@ -7664,10 +7664,10 @@
         <v>5478</v>
       </c>
       <c r="B320" t="n">
-        <v>1856.89995560344</v>
+        <v>1856.899955603444</v>
       </c>
       <c r="C320" t="n">
-        <v>6675.13939480431</v>
+        <v>6675.139394804326</v>
       </c>
     </row>
     <row r="321">
@@ -7675,10 +7675,10 @@
         <v>5479</v>
       </c>
       <c r="B321" t="n">
-        <v>12379.33303735631</v>
+        <v>12379.33303735647</v>
       </c>
       <c r="C321" t="n">
-        <v>44500.92929869557</v>
+        <v>44500.92929869613</v>
       </c>
     </row>
     <row r="322">
@@ -7829,10 +7829,10 @@
         <v>5493</v>
       </c>
       <c r="B335" t="n">
-        <v>1890.661705562905</v>
+        <v>1856.899955603447</v>
       </c>
       <c r="C335" t="n">
-        <v>6796.505323276597</v>
+        <v>6675.139394804335</v>
       </c>
     </row>
     <row r="336">
@@ -7840,10 +7840,10 @@
         <v>5494</v>
       </c>
       <c r="B336" t="n">
-        <v>0</v>
+        <v>1856.899955603429</v>
       </c>
       <c r="C336" t="n">
-        <v>0</v>
+        <v>6675.139394804271</v>
       </c>
     </row>
     <row r="337">
@@ -7854,7 +7854,7 @@
         <v>1856.899955603446</v>
       </c>
       <c r="C337" t="n">
-        <v>6675.139394804332</v>
+        <v>6675.139394804333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>